<commit_message>
Vehicle list: 13 brands, 89 models from official Thai brand sites
Gemini research (2026-09-27), reviewed by Core: brands, models, body
types, powertrains and years. Existing model ids kept (live URLs).
Dropped rows not confidently sold in Thailand as listed (Isuzu V-Cross
trim, Xforce HEV, Mazda6e, Tank ICE). Twin-powertrain models labelled
(e.g. 'City Hybrid'). newPrice is indicative and unverified; it only
feeds estimated values, hidden while SHOW_PRICES is off.

Engine tests pin the test car's price so data updates don't break them;
seed SQL and import template/example regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/examples/product-import-example.xlsx
+++ b/docs/examples/product-import-example.xlsx
@@ -568,7 +568,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="636" uniqueCount="258">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1154" uniqueCount="428">
   <si>
     <t>Unlimit Insure — แม่แบบนำเข้าข้อมูลแพ็กเกจ</t>
   </si>
@@ -1047,7 +1047,7 @@
     <t>toyota-yaris-ativ</t>
   </si>
   <si>
-    <t>Yaris Ativ</t>
+    <t>Yaris ATIV</t>
   </si>
   <si>
     <t>sedan</t>
@@ -1056,18 +1056,51 @@
     <t>ICE</t>
   </si>
   <si>
+    <t>toyota-yaris</t>
+  </si>
+  <si>
+    <t>Yaris</t>
+  </si>
+  <si>
+    <t>hatchback</t>
+  </si>
+  <si>
+    <t>toyota-yaris-cross-hev</t>
+  </si>
+  <si>
+    <t>Yaris Cross</t>
+  </si>
+  <si>
+    <t>suv</t>
+  </si>
+  <si>
+    <t>HEV</t>
+  </si>
+  <si>
+    <t>toyota-corolla-altis-ice</t>
+  </si>
+  <si>
+    <t>Corolla Altis</t>
+  </si>
+  <si>
+    <t>toyota-corolla-altis-hev</t>
+  </si>
+  <si>
+    <t>Corolla Altis Hybrid</t>
+  </si>
+  <si>
+    <t>toyota-camry-hev</t>
+  </si>
+  <si>
+    <t>Camry</t>
+  </si>
+  <si>
     <t>toyota-corolla-cross</t>
   </si>
   <si>
     <t>Corolla Cross</t>
   </si>
   <si>
-    <t>suv</t>
-  </si>
-  <si>
-    <t>HEV</t>
-  </si>
-  <si>
     <t>toyota-fortuner</t>
   </si>
   <si>
@@ -1083,6 +1116,36 @@
     <t>pickup</t>
   </si>
   <si>
+    <t>toyota-hilux-champ</t>
+  </si>
+  <si>
+    <t>Hilux Champ</t>
+  </si>
+  <si>
+    <t>toyota-veloz</t>
+  </si>
+  <si>
+    <t>Veloz</t>
+  </si>
+  <si>
+    <t>mpv</t>
+  </si>
+  <si>
+    <t>toyota-innova-zenix-hev</t>
+  </si>
+  <si>
+    <t>Innova Zenix</t>
+  </si>
+  <si>
+    <t>toyota-bz4x-ev</t>
+  </si>
+  <si>
+    <t>bZ4X</t>
+  </si>
+  <si>
+    <t>EV</t>
+  </si>
+  <si>
     <t>honda</t>
   </si>
   <si>
@@ -1098,6 +1161,24 @@
     <t>City</t>
   </si>
   <si>
+    <t>honda-city-hev</t>
+  </si>
+  <si>
+    <t>City Hybrid</t>
+  </si>
+  <si>
+    <t>honda-city-hatchback-ice</t>
+  </si>
+  <si>
+    <t>City Hatchback</t>
+  </si>
+  <si>
+    <t>honda-city-hatchback-hev</t>
+  </si>
+  <si>
+    <t>City Hatchback Hybrid</t>
+  </si>
+  <si>
     <t>honda-civic</t>
   </si>
   <si>
@@ -1107,7 +1188,37 @@
     <t>honda-hr-v</t>
   </si>
   <si>
-    <t>HR-V e:HEV</t>
+    <t>HR-V</t>
+  </si>
+  <si>
+    <t>honda-cr-v-ice</t>
+  </si>
+  <si>
+    <t>CR-V</t>
+  </si>
+  <si>
+    <t>honda-cr-v-hev</t>
+  </si>
+  <si>
+    <t>CR-V Hybrid</t>
+  </si>
+  <si>
+    <t>honda-accord-hev</t>
+  </si>
+  <si>
+    <t>Accord</t>
+  </si>
+  <si>
+    <t>honda-br-v</t>
+  </si>
+  <si>
+    <t>BR-V</t>
+  </si>
+  <si>
+    <t>honda-e-n1-ev</t>
+  </si>
+  <si>
+    <t>e:N1</t>
   </si>
   <si>
     <t>isuzu</t>
@@ -1125,6 +1236,90 @@
     <t>D-Max</t>
   </si>
   <si>
+    <t>isuzu-mu-x</t>
+  </si>
+  <si>
+    <t>MU-X</t>
+  </si>
+  <si>
+    <t>mitsubishi</t>
+  </si>
+  <si>
+    <t>Mitsubishi</t>
+  </si>
+  <si>
+    <t>มิตซูบิชิ</t>
+  </si>
+  <si>
+    <t>mitsubishi-mirage</t>
+  </si>
+  <si>
+    <t>Mirage</t>
+  </si>
+  <si>
+    <t>mitsubishi-attrage</t>
+  </si>
+  <si>
+    <t>Attrage</t>
+  </si>
+  <si>
+    <t>mitsubishi-xpander-hev</t>
+  </si>
+  <si>
+    <t>Xpander</t>
+  </si>
+  <si>
+    <t>mitsubishi-xpander-cross-hev</t>
+  </si>
+  <si>
+    <t>Xpander Cross</t>
+  </si>
+  <si>
+    <t>mitsubishi-pajero-sport</t>
+  </si>
+  <si>
+    <t>Pajero Sport</t>
+  </si>
+  <si>
+    <t>mitsubishi-triton</t>
+  </si>
+  <si>
+    <t>Triton</t>
+  </si>
+  <si>
+    <t>nissan</t>
+  </si>
+  <si>
+    <t>Nissan</t>
+  </si>
+  <si>
+    <t>นิสสัน</t>
+  </si>
+  <si>
+    <t>nissan-almera</t>
+  </si>
+  <si>
+    <t>Almera</t>
+  </si>
+  <si>
+    <t>nissan-kicks-hev</t>
+  </si>
+  <si>
+    <t>Kicks e-POWER</t>
+  </si>
+  <si>
+    <t>nissan-navara</t>
+  </si>
+  <si>
+    <t>Navara</t>
+  </si>
+  <si>
+    <t>nissan-terra</t>
+  </si>
+  <si>
+    <t>Terra</t>
+  </si>
+  <si>
     <t>mazda</t>
   </si>
   <si>
@@ -1134,13 +1329,40 @@
     <t>มาสด้า</t>
   </si>
   <si>
+    <t>mazda-2-sedan</t>
+  </si>
+  <si>
+    <t>Mazda2 Sedan</t>
+  </si>
+  <si>
     <t>mazda-2</t>
   </si>
   <si>
-    <t>Mazda2</t>
-  </si>
-  <si>
-    <t>hatchback</t>
+    <t>Mazda2 Hatchback</t>
+  </si>
+  <si>
+    <t>mazda-3-sedan</t>
+  </si>
+  <si>
+    <t>Mazda3 Sedan</t>
+  </si>
+  <si>
+    <t>mazda-3-fastback</t>
+  </si>
+  <si>
+    <t>Mazda3 Fastback</t>
+  </si>
+  <si>
+    <t>mazda-cx-3</t>
+  </si>
+  <si>
+    <t>CX-3</t>
+  </si>
+  <si>
+    <t>mazda-cx-30</t>
+  </si>
+  <si>
+    <t>CX-30</t>
   </si>
   <si>
     <t>mazda-cx-5</t>
@@ -1149,6 +1371,129 @@
     <t>CX-5</t>
   </si>
   <si>
+    <t>mazda-cx-8</t>
+  </si>
+  <si>
+    <t>CX-8</t>
+  </si>
+  <si>
+    <t>mazda-bt-50</t>
+  </si>
+  <si>
+    <t>BT-50</t>
+  </si>
+  <si>
+    <t>ford</t>
+  </si>
+  <si>
+    <t>Ford</t>
+  </si>
+  <si>
+    <t>ฟอร์ด</t>
+  </si>
+  <si>
+    <t>ford-ranger</t>
+  </si>
+  <si>
+    <t>Ranger</t>
+  </si>
+  <si>
+    <t>ford-ranger-raptor</t>
+  </si>
+  <si>
+    <t>Ranger Raptor</t>
+  </si>
+  <si>
+    <t>ford-everest</t>
+  </si>
+  <si>
+    <t>Everest</t>
+  </si>
+  <si>
+    <t>mg</t>
+  </si>
+  <si>
+    <t>MG</t>
+  </si>
+  <si>
+    <t>เอ็มจี</t>
+  </si>
+  <si>
+    <t>mg-3-hev</t>
+  </si>
+  <si>
+    <t>MG3 Hybrid+</t>
+  </si>
+  <si>
+    <t>mg-5</t>
+  </si>
+  <si>
+    <t>MG5</t>
+  </si>
+  <si>
+    <t>mg-zs</t>
+  </si>
+  <si>
+    <t>MG ZS</t>
+  </si>
+  <si>
+    <t>mg-zs-ev</t>
+  </si>
+  <si>
+    <t>MG ZS EV</t>
+  </si>
+  <si>
+    <t>mg-vs-hev</t>
+  </si>
+  <si>
+    <t>MG VS HEV</t>
+  </si>
+  <si>
+    <t>mg-hs-phev</t>
+  </si>
+  <si>
+    <t>MG HS PHEV</t>
+  </si>
+  <si>
+    <t>PHEV</t>
+  </si>
+  <si>
+    <t>mg-4</t>
+  </si>
+  <si>
+    <t>MG4 Electric</t>
+  </si>
+  <si>
+    <t>mg-ep-ev</t>
+  </si>
+  <si>
+    <t>MG EP Plus</t>
+  </si>
+  <si>
+    <t>mg-es-ev</t>
+  </si>
+  <si>
+    <t>MG ES</t>
+  </si>
+  <si>
+    <t>mg-maxus-7-ev</t>
+  </si>
+  <si>
+    <t>MG Maxus 7</t>
+  </si>
+  <si>
+    <t>mg-maxus-9-ev</t>
+  </si>
+  <si>
+    <t>MG Maxus 9</t>
+  </si>
+  <si>
+    <t>mg-extender</t>
+  </si>
+  <si>
+    <t>MG Extender</t>
+  </si>
+  <si>
     <t>byd</t>
   </si>
   <si>
@@ -1164,43 +1509,208 @@
     <t>Dolphin</t>
   </si>
   <si>
-    <t>EV</t>
-  </si>
-  <si>
     <t>byd-atto-3</t>
   </si>
   <si>
     <t>Atto 3</t>
   </si>
   <si>
+    <t>byd-seal-ev</t>
+  </si>
+  <si>
+    <t>Seal</t>
+  </si>
+  <si>
     <t>byd-sealion-6</t>
   </si>
   <si>
-    <t>Sealion 6</t>
-  </si>
-  <si>
-    <t>PHEV</t>
-  </si>
-  <si>
-    <t>mg</t>
-  </si>
-  <si>
-    <t>MG</t>
-  </si>
-  <si>
-    <t>เอ็มจี</t>
-  </si>
-  <si>
-    <t>mg-zs-ev</t>
-  </si>
-  <si>
-    <t>ZS EV</t>
-  </si>
-  <si>
-    <t>mg-4</t>
-  </si>
-  <si>
-    <t>MG4 Electric</t>
+    <t>Sealion 6 DM-i</t>
+  </si>
+  <si>
+    <t>byd-m6-ev</t>
+  </si>
+  <si>
+    <t>M6</t>
+  </si>
+  <si>
+    <t>byd-sealion-7-ev</t>
+  </si>
+  <si>
+    <t>Sealion 7</t>
+  </si>
+  <si>
+    <t>suzuki</t>
+  </si>
+  <si>
+    <t>Suzuki</t>
+  </si>
+  <si>
+    <t>ซูซูกิ</t>
+  </si>
+  <si>
+    <t>suzuki-celerio</t>
+  </si>
+  <si>
+    <t>Celerio</t>
+  </si>
+  <si>
+    <t>suzuki-swift</t>
+  </si>
+  <si>
+    <t>Swift</t>
+  </si>
+  <si>
+    <t>suzuki-xl7-hev</t>
+  </si>
+  <si>
+    <t>XL7 Hybrid</t>
+  </si>
+  <si>
+    <t>suzuki-carry</t>
+  </si>
+  <si>
+    <t>Carry</t>
+  </si>
+  <si>
+    <t>suzuki-jimny</t>
+  </si>
+  <si>
+    <t>Jimny</t>
+  </si>
+  <si>
+    <t>gwm</t>
+  </si>
+  <si>
+    <t>GWM</t>
+  </si>
+  <si>
+    <t>เกรท วอลล์ มอเตอร์</t>
+  </si>
+  <si>
+    <t>gwm-haval-h6-hev</t>
+  </si>
+  <si>
+    <t>Haval H6 Hybrid</t>
+  </si>
+  <si>
+    <t>gwm-haval-h6-phev</t>
+  </si>
+  <si>
+    <t>Haval H6</t>
+  </si>
+  <si>
+    <t>gwm-ora-good-cat-ev</t>
+  </si>
+  <si>
+    <t>ORA Good Cat</t>
+  </si>
+  <si>
+    <t>gwm-ora-07-ev</t>
+  </si>
+  <si>
+    <t>ORA 07</t>
+  </si>
+  <si>
+    <t>gwm-ora-5-ev</t>
+  </si>
+  <si>
+    <t>ORA 5 EV</t>
+  </si>
+  <si>
+    <t>gwm-ora-5-hev</t>
+  </si>
+  <si>
+    <t>ORA 5</t>
+  </si>
+  <si>
+    <t>gwm-tank-300-hev</t>
+  </si>
+  <si>
+    <t>Tank 300</t>
+  </si>
+  <si>
+    <t>gwm-tank-500-hev</t>
+  </si>
+  <si>
+    <t>Tank 500</t>
+  </si>
+  <si>
+    <t>gwm-poer-sahar-hev</t>
+  </si>
+  <si>
+    <t>Poer Sahar</t>
+  </si>
+  <si>
+    <t>hyundai</t>
+  </si>
+  <si>
+    <t>Hyundai</t>
+  </si>
+  <si>
+    <t>ฮุนได</t>
+  </si>
+  <si>
+    <t>hyundai-creta</t>
+  </si>
+  <si>
+    <t>Creta</t>
+  </si>
+  <si>
+    <t>hyundai-stargazer</t>
+  </si>
+  <si>
+    <t>Stargazer</t>
+  </si>
+  <si>
+    <t>hyundai-staria-ice</t>
+  </si>
+  <si>
+    <t>Staria</t>
+  </si>
+  <si>
+    <t>hyundai-staria-hev</t>
+  </si>
+  <si>
+    <t>Staria Hybrid</t>
+  </si>
+  <si>
+    <t>hyundai-santa-fe-hev</t>
+  </si>
+  <si>
+    <t>Santa Fe</t>
+  </si>
+  <si>
+    <t>hyundai-ioniq-5-ev</t>
+  </si>
+  <si>
+    <t>Ioniq 5</t>
+  </si>
+  <si>
+    <t>hyundai-palisade</t>
+  </si>
+  <si>
+    <t>Palisade</t>
+  </si>
+  <si>
+    <t>tesla</t>
+  </si>
+  <si>
+    <t>Tesla</t>
+  </si>
+  <si>
+    <t>เทสลา</t>
+  </si>
+  <si>
+    <t>tesla-model-3-ev</t>
+  </si>
+  <si>
+    <t>Model 3</t>
+  </si>
+  <si>
+    <t>tesla-model-y-ev</t>
+  </si>
+  <si>
+    <t>Model Y</t>
   </si>
   <si>
     <t>a-type1-dealer</t>
@@ -2932,10 +3442,10 @@
         <v>161</v>
       </c>
       <c r="H2">
-        <v>600000</v>
+        <v>569000</v>
       </c>
       <c r="I2">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="J2">
         <v>2026</v>
@@ -2961,13 +3471,13 @@
         <v>164</v>
       </c>
       <c r="G3" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="H3">
-        <v>1050000</v>
+        <v>584000</v>
       </c>
       <c r="I3">
-        <v>2020</v>
+        <v>2015</v>
       </c>
       <c r="J3">
         <v>2026</v>
@@ -2984,22 +3494,22 @@
         <v>157</v>
       </c>
       <c r="D4" t="s">
+        <v>165</v>
+      </c>
+      <c r="E4" t="s">
         <v>166</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>167</v>
       </c>
-      <c r="F4" t="s">
-        <v>164</v>
-      </c>
       <c r="G4" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="H4">
-        <v>1500000</v>
+        <v>809000</v>
       </c>
       <c r="I4">
-        <v>2019</v>
+        <v>2023</v>
       </c>
       <c r="J4">
         <v>2026</v>
@@ -3016,19 +3526,19 @@
         <v>157</v>
       </c>
       <c r="D5" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F5" t="s">
-        <v>170</v>
+        <v>160</v>
       </c>
       <c r="G5" t="s">
         <v>161</v>
       </c>
       <c r="H5">
-        <v>800000</v>
+        <v>909000</v>
       </c>
       <c r="I5">
         <v>2019</v>
@@ -3039,31 +3549,31 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>155</v>
+      </c>
+      <c r="B6" t="s">
+        <v>156</v>
+      </c>
+      <c r="C6" t="s">
+        <v>157</v>
+      </c>
+      <c r="D6" t="s">
         <v>171</v>
       </c>
-      <c r="B6" t="s">
+      <c r="E6" t="s">
         <v>172</v>
-      </c>
-      <c r="C6" t="s">
-        <v>173</v>
-      </c>
-      <c r="D6" t="s">
-        <v>174</v>
-      </c>
-      <c r="E6" t="s">
-        <v>175</v>
       </c>
       <c r="F6" t="s">
         <v>160</v>
       </c>
       <c r="G6" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="H6">
-        <v>620000</v>
+        <v>909000</v>
       </c>
       <c r="I6">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="J6">
         <v>2026</v>
@@ -3071,31 +3581,31 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>171</v>
+        <v>155</v>
       </c>
       <c r="B7" t="s">
-        <v>172</v>
+        <v>156</v>
       </c>
       <c r="C7" t="s">
+        <v>157</v>
+      </c>
+      <c r="D7" t="s">
         <v>173</v>
       </c>
-      <c r="D7" t="s">
-        <v>176</v>
-      </c>
       <c r="E7" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="F7" t="s">
         <v>160</v>
       </c>
       <c r="G7" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="H7">
-        <v>1000000</v>
+        <v>1475000</v>
       </c>
       <c r="I7">
-        <v>2021</v>
+        <v>2018</v>
       </c>
       <c r="J7">
         <v>2026</v>
@@ -3103,31 +3613,31 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>171</v>
+        <v>155</v>
       </c>
       <c r="B8" t="s">
-        <v>172</v>
+        <v>156</v>
       </c>
       <c r="C8" t="s">
-        <v>173</v>
+        <v>157</v>
       </c>
       <c r="D8" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="E8" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="F8" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="G8" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="H8">
-        <v>1100000</v>
+        <v>989000</v>
       </c>
       <c r="I8">
-        <v>2022</v>
+        <v>2020</v>
       </c>
       <c r="J8">
         <v>2026</v>
@@ -3135,31 +3645,31 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>180</v>
+        <v>155</v>
       </c>
       <c r="B9" t="s">
-        <v>181</v>
+        <v>156</v>
       </c>
       <c r="C9" t="s">
-        <v>182</v>
+        <v>157</v>
       </c>
       <c r="D9" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="E9" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="F9" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="G9" t="s">
         <v>161</v>
       </c>
       <c r="H9">
-        <v>750000</v>
+        <v>1239000</v>
       </c>
       <c r="I9">
-        <v>2019</v>
+        <v>2015</v>
       </c>
       <c r="J9">
         <v>2026</v>
@@ -3167,31 +3677,31 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>185</v>
+        <v>155</v>
       </c>
       <c r="B10" t="s">
-        <v>186</v>
+        <v>156</v>
       </c>
       <c r="C10" t="s">
-        <v>187</v>
+        <v>157</v>
       </c>
       <c r="D10" t="s">
-        <v>188</v>
+        <v>179</v>
       </c>
       <c r="E10" t="s">
-        <v>189</v>
+        <v>180</v>
       </c>
       <c r="F10" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="G10" t="s">
         <v>161</v>
       </c>
       <c r="H10">
-        <v>600000</v>
+        <v>554000</v>
       </c>
       <c r="I10">
-        <v>2019</v>
+        <v>2015</v>
       </c>
       <c r="J10">
         <v>2026</v>
@@ -3199,31 +3709,31 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>185</v>
+        <v>155</v>
       </c>
       <c r="B11" t="s">
-        <v>186</v>
+        <v>156</v>
       </c>
       <c r="C11" t="s">
-        <v>187</v>
+        <v>157</v>
       </c>
       <c r="D11" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
       <c r="E11" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
       <c r="F11" t="s">
-        <v>164</v>
+        <v>181</v>
       </c>
       <c r="G11" t="s">
         <v>161</v>
       </c>
       <c r="H11">
-        <v>1300000</v>
+        <v>459000</v>
       </c>
       <c r="I11">
-        <v>2019</v>
+        <v>2023</v>
       </c>
       <c r="J11">
         <v>2026</v>
@@ -3231,31 +3741,31 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>193</v>
+        <v>155</v>
       </c>
       <c r="B12" t="s">
-        <v>194</v>
+        <v>156</v>
       </c>
       <c r="C12" t="s">
-        <v>195</v>
+        <v>157</v>
       </c>
       <c r="D12" t="s">
-        <v>196</v>
+        <v>184</v>
       </c>
       <c r="E12" t="s">
-        <v>197</v>
+        <v>185</v>
       </c>
       <c r="F12" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="G12" t="s">
-        <v>198</v>
+        <v>161</v>
       </c>
       <c r="H12">
-        <v>700000</v>
+        <v>795000</v>
       </c>
       <c r="I12">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="J12">
         <v>2026</v>
@@ -3263,31 +3773,31 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>193</v>
+        <v>155</v>
       </c>
       <c r="B13" t="s">
-        <v>194</v>
+        <v>156</v>
       </c>
       <c r="C13" t="s">
-        <v>195</v>
+        <v>157</v>
       </c>
       <c r="D13" t="s">
-        <v>199</v>
+        <v>187</v>
       </c>
       <c r="E13" t="s">
-        <v>200</v>
+        <v>188</v>
       </c>
       <c r="F13" t="s">
-        <v>164</v>
+        <v>186</v>
       </c>
       <c r="G13" t="s">
-        <v>198</v>
+        <v>168</v>
       </c>
       <c r="H13">
-        <v>1000000</v>
+        <v>1379000</v>
       </c>
       <c r="I13">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="J13">
         <v>2026</v>
@@ -3295,31 +3805,31 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>193</v>
+        <v>155</v>
       </c>
       <c r="B14" t="s">
-        <v>194</v>
+        <v>156</v>
       </c>
       <c r="C14" t="s">
-        <v>195</v>
+        <v>157</v>
       </c>
       <c r="D14" t="s">
-        <v>201</v>
+        <v>189</v>
       </c>
       <c r="E14" t="s">
-        <v>202</v>
+        <v>190</v>
       </c>
       <c r="F14" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="G14" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
       <c r="H14">
-        <v>1100000</v>
+        <v>1529000</v>
       </c>
       <c r="I14">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="J14">
         <v>2026</v>
@@ -3327,31 +3837,31 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
       <c r="B15" t="s">
-        <v>205</v>
+        <v>193</v>
       </c>
       <c r="C15" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
       <c r="D15" t="s">
-        <v>207</v>
+        <v>195</v>
       </c>
       <c r="E15" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="F15" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="G15" t="s">
-        <v>198</v>
+        <v>161</v>
       </c>
       <c r="H15">
-        <v>900000</v>
+        <v>569000</v>
       </c>
       <c r="I15">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="J15">
         <v>2026</v>
@@ -3359,110 +3869,2404 @@
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>192</v>
+      </c>
+      <c r="B16" t="s">
+        <v>193</v>
+      </c>
+      <c r="C16" t="s">
+        <v>194</v>
+      </c>
+      <c r="D16" t="s">
+        <v>197</v>
+      </c>
+      <c r="E16" t="s">
+        <v>198</v>
+      </c>
+      <c r="F16" t="s">
+        <v>160</v>
+      </c>
+      <c r="G16" t="s">
+        <v>168</v>
+      </c>
+      <c r="H16">
+        <v>729000</v>
+      </c>
+      <c r="I16">
+        <v>2020</v>
+      </c>
+      <c r="J16">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>192</v>
+      </c>
+      <c r="B17" t="s">
+        <v>193</v>
+      </c>
+      <c r="C17" t="s">
+        <v>194</v>
+      </c>
+      <c r="D17" t="s">
+        <v>199</v>
+      </c>
+      <c r="E17" t="s">
+        <v>200</v>
+      </c>
+      <c r="F17" t="s">
+        <v>164</v>
+      </c>
+      <c r="G17" t="s">
+        <v>161</v>
+      </c>
+      <c r="H17">
+        <v>599000</v>
+      </c>
+      <c r="I17">
+        <v>2020</v>
+      </c>
+      <c r="J17">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>192</v>
+      </c>
+      <c r="B18" t="s">
+        <v>193</v>
+      </c>
+      <c r="C18" t="s">
+        <v>194</v>
+      </c>
+      <c r="D18" t="s">
+        <v>201</v>
+      </c>
+      <c r="E18" t="s">
+        <v>202</v>
+      </c>
+      <c r="F18" t="s">
+        <v>164</v>
+      </c>
+      <c r="G18" t="s">
+        <v>168</v>
+      </c>
+      <c r="H18">
+        <v>729000</v>
+      </c>
+      <c r="I18">
+        <v>2021</v>
+      </c>
+      <c r="J18">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>192</v>
+      </c>
+      <c r="B19" t="s">
+        <v>193</v>
+      </c>
+      <c r="C19" t="s">
+        <v>194</v>
+      </c>
+      <c r="D19" t="s">
+        <v>203</v>
+      </c>
+      <c r="E19" t="s">
         <v>204</v>
       </c>
-      <c r="B16" t="s">
+      <c r="F19" t="s">
+        <v>160</v>
+      </c>
+      <c r="G19" t="s">
+        <v>168</v>
+      </c>
+      <c r="H19">
+        <v>949000</v>
+      </c>
+      <c r="I19">
+        <v>2022</v>
+      </c>
+      <c r="J19">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>192</v>
+      </c>
+      <c r="B20" t="s">
+        <v>193</v>
+      </c>
+      <c r="C20" t="s">
+        <v>194</v>
+      </c>
+      <c r="D20" t="s">
         <v>205</v>
       </c>
-      <c r="C16" t="s">
+      <c r="E20" t="s">
         <v>206</v>
       </c>
-      <c r="D16" t="s">
+      <c r="F20" t="s">
+        <v>167</v>
+      </c>
+      <c r="G20" t="s">
+        <v>168</v>
+      </c>
+      <c r="H20">
+        <v>899000</v>
+      </c>
+      <c r="I20">
+        <v>2021</v>
+      </c>
+      <c r="J20">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>192</v>
+      </c>
+      <c r="B21" t="s">
+        <v>193</v>
+      </c>
+      <c r="C21" t="s">
+        <v>194</v>
+      </c>
+      <c r="D21" t="s">
+        <v>207</v>
+      </c>
+      <c r="E21" t="s">
+        <v>208</v>
+      </c>
+      <c r="F21" t="s">
+        <v>167</v>
+      </c>
+      <c r="G21" t="s">
+        <v>161</v>
+      </c>
+      <c r="H21">
+        <v>1419000</v>
+      </c>
+      <c r="I21">
+        <v>2023</v>
+      </c>
+      <c r="J21">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>192</v>
+      </c>
+      <c r="B22" t="s">
+        <v>193</v>
+      </c>
+      <c r="C22" t="s">
+        <v>194</v>
+      </c>
+      <c r="D22" t="s">
         <v>209</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E22" t="s">
         <v>210</v>
       </c>
-      <c r="F16" t="s">
-        <v>190</v>
-      </c>
-      <c r="G16" t="s">
-        <v>198</v>
-      </c>
-      <c r="H16">
-        <v>850000</v>
-      </c>
-      <c r="I16">
+      <c r="F22" t="s">
+        <v>167</v>
+      </c>
+      <c r="G22" t="s">
+        <v>168</v>
+      </c>
+      <c r="H22">
+        <v>1409000</v>
+      </c>
+      <c r="I22">
+        <v>2023</v>
+      </c>
+      <c r="J22">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>192</v>
+      </c>
+      <c r="B23" t="s">
+        <v>193</v>
+      </c>
+      <c r="C23" t="s">
+        <v>194</v>
+      </c>
+      <c r="D23" t="s">
+        <v>211</v>
+      </c>
+      <c r="E23" t="s">
+        <v>212</v>
+      </c>
+      <c r="F23" t="s">
+        <v>160</v>
+      </c>
+      <c r="G23" t="s">
+        <v>168</v>
+      </c>
+      <c r="H23">
+        <v>1529000</v>
+      </c>
+      <c r="I23">
+        <v>2023</v>
+      </c>
+      <c r="J23">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>192</v>
+      </c>
+      <c r="B24" t="s">
+        <v>193</v>
+      </c>
+      <c r="C24" t="s">
+        <v>194</v>
+      </c>
+      <c r="D24" t="s">
+        <v>213</v>
+      </c>
+      <c r="E24" t="s">
+        <v>214</v>
+      </c>
+      <c r="F24" t="s">
+        <v>186</v>
+      </c>
+      <c r="G24" t="s">
+        <v>161</v>
+      </c>
+      <c r="H24">
+        <v>915000</v>
+      </c>
+      <c r="I24">
         <v>2022</v>
       </c>
-      <c r="J16">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="17" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="18" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="19" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="20" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="21" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="22" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="23" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="24" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="25" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="26" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="27" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="29" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="30" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="31" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="32" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="33" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="34" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="35" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="36" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="37" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="38" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="39" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="40" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="41" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="42" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="43" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="44" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="45" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="46" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="47" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="48" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="49" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="50" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="51" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="52" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="53" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="54" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="55" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="56" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="57" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="58" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="59" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="60" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="61" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="62" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="63" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="64" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="65" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="66" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="67" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="68" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="69" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="70" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="71" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="72" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="73" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="74" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="75" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="76" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="77" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="78" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="79" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="80" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="81" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="82" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="83" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="84" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="85" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="86" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="87" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="88" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="89" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="90" spans="6:7" x14ac:dyDescent="0.25"/>
+      <c r="J24">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>192</v>
+      </c>
+      <c r="B25" t="s">
+        <v>193</v>
+      </c>
+      <c r="C25" t="s">
+        <v>194</v>
+      </c>
+      <c r="D25" t="s">
+        <v>215</v>
+      </c>
+      <c r="E25" t="s">
+        <v>216</v>
+      </c>
+      <c r="F25" t="s">
+        <v>167</v>
+      </c>
+      <c r="G25" t="s">
+        <v>191</v>
+      </c>
+      <c r="H25">
+        <v>1199000</v>
+      </c>
+      <c r="I25">
+        <v>2024</v>
+      </c>
+      <c r="J25">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>217</v>
+      </c>
+      <c r="B26" t="s">
+        <v>218</v>
+      </c>
+      <c r="C26" t="s">
+        <v>219</v>
+      </c>
+      <c r="D26" t="s">
+        <v>220</v>
+      </c>
+      <c r="E26" t="s">
+        <v>221</v>
+      </c>
+      <c r="F26" t="s">
+        <v>181</v>
+      </c>
+      <c r="G26" t="s">
+        <v>161</v>
+      </c>
+      <c r="H26">
+        <v>552000</v>
+      </c>
+      <c r="I26">
+        <v>2019</v>
+      </c>
+      <c r="J26">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>217</v>
+      </c>
+      <c r="B27" t="s">
+        <v>218</v>
+      </c>
+      <c r="C27" t="s">
+        <v>219</v>
+      </c>
+      <c r="D27" t="s">
+        <v>222</v>
+      </c>
+      <c r="E27" t="s">
+        <v>223</v>
+      </c>
+      <c r="F27" t="s">
+        <v>167</v>
+      </c>
+      <c r="G27" t="s">
+        <v>161</v>
+      </c>
+      <c r="H27">
+        <v>1184000</v>
+      </c>
+      <c r="I27">
+        <v>2020</v>
+      </c>
+      <c r="J27">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>224</v>
+      </c>
+      <c r="B28" t="s">
+        <v>225</v>
+      </c>
+      <c r="C28" t="s">
+        <v>226</v>
+      </c>
+      <c r="D28" t="s">
+        <v>227</v>
+      </c>
+      <c r="E28" t="s">
+        <v>228</v>
+      </c>
+      <c r="F28" t="s">
+        <v>164</v>
+      </c>
+      <c r="G28" t="s">
+        <v>161</v>
+      </c>
+      <c r="H28">
+        <v>509000</v>
+      </c>
+      <c r="I28">
+        <v>2015</v>
+      </c>
+      <c r="J28">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>224</v>
+      </c>
+      <c r="B29" t="s">
+        <v>225</v>
+      </c>
+      <c r="C29" t="s">
+        <v>226</v>
+      </c>
+      <c r="D29" t="s">
+        <v>229</v>
+      </c>
+      <c r="E29" t="s">
+        <v>230</v>
+      </c>
+      <c r="F29" t="s">
+        <v>160</v>
+      </c>
+      <c r="G29" t="s">
+        <v>161</v>
+      </c>
+      <c r="H29">
+        <v>519000</v>
+      </c>
+      <c r="I29">
+        <v>2015</v>
+      </c>
+      <c r="J29">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>224</v>
+      </c>
+      <c r="B30" t="s">
+        <v>225</v>
+      </c>
+      <c r="C30" t="s">
+        <v>226</v>
+      </c>
+      <c r="D30" t="s">
+        <v>231</v>
+      </c>
+      <c r="E30" t="s">
+        <v>232</v>
+      </c>
+      <c r="F30" t="s">
+        <v>186</v>
+      </c>
+      <c r="G30" t="s">
+        <v>168</v>
+      </c>
+      <c r="H30">
+        <v>939000</v>
+      </c>
+      <c r="I30">
+        <v>2024</v>
+      </c>
+      <c r="J30">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>224</v>
+      </c>
+      <c r="B31" t="s">
+        <v>225</v>
+      </c>
+      <c r="C31" t="s">
+        <v>226</v>
+      </c>
+      <c r="D31" t="s">
+        <v>233</v>
+      </c>
+      <c r="E31" t="s">
+        <v>234</v>
+      </c>
+      <c r="F31" t="s">
+        <v>186</v>
+      </c>
+      <c r="G31" t="s">
+        <v>168</v>
+      </c>
+      <c r="H31">
+        <v>969000</v>
+      </c>
+      <c r="I31">
+        <v>2024</v>
+      </c>
+      <c r="J31">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>224</v>
+      </c>
+      <c r="B32" t="s">
+        <v>225</v>
+      </c>
+      <c r="C32" t="s">
+        <v>226</v>
+      </c>
+      <c r="D32" t="s">
+        <v>235</v>
+      </c>
+      <c r="E32" t="s">
+        <v>236</v>
+      </c>
+      <c r="F32" t="s">
+        <v>167</v>
+      </c>
+      <c r="G32" t="s">
+        <v>161</v>
+      </c>
+      <c r="H32">
+        <v>1139000</v>
+      </c>
+      <c r="I32">
+        <v>2015</v>
+      </c>
+      <c r="J32">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>224</v>
+      </c>
+      <c r="B33" t="s">
+        <v>225</v>
+      </c>
+      <c r="C33" t="s">
+        <v>226</v>
+      </c>
+      <c r="D33" t="s">
+        <v>237</v>
+      </c>
+      <c r="E33" t="s">
+        <v>238</v>
+      </c>
+      <c r="F33" t="s">
+        <v>181</v>
+      </c>
+      <c r="G33" t="s">
+        <v>161</v>
+      </c>
+      <c r="H33">
+        <v>614000</v>
+      </c>
+      <c r="I33">
+        <v>2023</v>
+      </c>
+      <c r="J33">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>239</v>
+      </c>
+      <c r="B34" t="s">
+        <v>240</v>
+      </c>
+      <c r="C34" t="s">
+        <v>241</v>
+      </c>
+      <c r="D34" t="s">
+        <v>242</v>
+      </c>
+      <c r="E34" t="s">
+        <v>243</v>
+      </c>
+      <c r="F34" t="s">
+        <v>160</v>
+      </c>
+      <c r="G34" t="s">
+        <v>161</v>
+      </c>
+      <c r="H34">
+        <v>549000</v>
+      </c>
+      <c r="I34">
+        <v>2019</v>
+      </c>
+      <c r="J34">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>239</v>
+      </c>
+      <c r="B35" t="s">
+        <v>240</v>
+      </c>
+      <c r="C35" t="s">
+        <v>241</v>
+      </c>
+      <c r="D35" t="s">
+        <v>244</v>
+      </c>
+      <c r="E35" t="s">
+        <v>245</v>
+      </c>
+      <c r="F35" t="s">
+        <v>167</v>
+      </c>
+      <c r="G35" t="s">
+        <v>168</v>
+      </c>
+      <c r="H35">
+        <v>789900</v>
+      </c>
+      <c r="I35">
+        <v>2020</v>
+      </c>
+      <c r="J35">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>239</v>
+      </c>
+      <c r="B36" t="s">
+        <v>240</v>
+      </c>
+      <c r="C36" t="s">
+        <v>241</v>
+      </c>
+      <c r="D36" t="s">
+        <v>246</v>
+      </c>
+      <c r="E36" t="s">
+        <v>247</v>
+      </c>
+      <c r="F36" t="s">
+        <v>181</v>
+      </c>
+      <c r="G36" t="s">
+        <v>161</v>
+      </c>
+      <c r="H36">
+        <v>599000</v>
+      </c>
+      <c r="I36">
+        <v>2020</v>
+      </c>
+      <c r="J36">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>239</v>
+      </c>
+      <c r="B37" t="s">
+        <v>240</v>
+      </c>
+      <c r="C37" t="s">
+        <v>241</v>
+      </c>
+      <c r="D37" t="s">
+        <v>248</v>
+      </c>
+      <c r="E37" t="s">
+        <v>249</v>
+      </c>
+      <c r="F37" t="s">
+        <v>167</v>
+      </c>
+      <c r="G37" t="s">
+        <v>161</v>
+      </c>
+      <c r="H37">
+        <v>1199000</v>
+      </c>
+      <c r="I37">
+        <v>2018</v>
+      </c>
+      <c r="J37">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>250</v>
+      </c>
+      <c r="B38" t="s">
+        <v>251</v>
+      </c>
+      <c r="C38" t="s">
+        <v>252</v>
+      </c>
+      <c r="D38" t="s">
+        <v>253</v>
+      </c>
+      <c r="E38" t="s">
+        <v>254</v>
+      </c>
+      <c r="F38" t="s">
+        <v>160</v>
+      </c>
+      <c r="G38" t="s">
+        <v>161</v>
+      </c>
+      <c r="H38">
+        <v>529000</v>
+      </c>
+      <c r="I38">
+        <v>2015</v>
+      </c>
+      <c r="J38">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>250</v>
+      </c>
+      <c r="B39" t="s">
+        <v>251</v>
+      </c>
+      <c r="C39" t="s">
+        <v>252</v>
+      </c>
+      <c r="D39" t="s">
+        <v>255</v>
+      </c>
+      <c r="E39" t="s">
+        <v>256</v>
+      </c>
+      <c r="F39" t="s">
+        <v>164</v>
+      </c>
+      <c r="G39" t="s">
+        <v>161</v>
+      </c>
+      <c r="H39">
+        <v>529000</v>
+      </c>
+      <c r="I39">
+        <v>2015</v>
+      </c>
+      <c r="J39">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>250</v>
+      </c>
+      <c r="B40" t="s">
+        <v>251</v>
+      </c>
+      <c r="C40" t="s">
+        <v>252</v>
+      </c>
+      <c r="D40" t="s">
+        <v>257</v>
+      </c>
+      <c r="E40" t="s">
+        <v>258</v>
+      </c>
+      <c r="F40" t="s">
+        <v>160</v>
+      </c>
+      <c r="G40" t="s">
+        <v>161</v>
+      </c>
+      <c r="H40">
+        <v>979000</v>
+      </c>
+      <c r="I40">
+        <v>2019</v>
+      </c>
+      <c r="J40">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>250</v>
+      </c>
+      <c r="B41" t="s">
+        <v>251</v>
+      </c>
+      <c r="C41" t="s">
+        <v>252</v>
+      </c>
+      <c r="D41" t="s">
+        <v>259</v>
+      </c>
+      <c r="E41" t="s">
+        <v>260</v>
+      </c>
+      <c r="F41" t="s">
+        <v>164</v>
+      </c>
+      <c r="G41" t="s">
+        <v>161</v>
+      </c>
+      <c r="H41">
+        <v>979000</v>
+      </c>
+      <c r="I41">
+        <v>2019</v>
+      </c>
+      <c r="J41">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>250</v>
+      </c>
+      <c r="B42" t="s">
+        <v>251</v>
+      </c>
+      <c r="C42" t="s">
+        <v>252</v>
+      </c>
+      <c r="D42" t="s">
+        <v>261</v>
+      </c>
+      <c r="E42" t="s">
+        <v>262</v>
+      </c>
+      <c r="F42" t="s">
+        <v>167</v>
+      </c>
+      <c r="G42" t="s">
+        <v>161</v>
+      </c>
+      <c r="H42">
+        <v>699000</v>
+      </c>
+      <c r="I42">
+        <v>2015</v>
+      </c>
+      <c r="J42">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>250</v>
+      </c>
+      <c r="B43" t="s">
+        <v>251</v>
+      </c>
+      <c r="C43" t="s">
+        <v>252</v>
+      </c>
+      <c r="D43" t="s">
+        <v>263</v>
+      </c>
+      <c r="E43" t="s">
+        <v>264</v>
+      </c>
+      <c r="F43" t="s">
+        <v>167</v>
+      </c>
+      <c r="G43" t="s">
+        <v>161</v>
+      </c>
+      <c r="H43">
+        <v>899000</v>
+      </c>
+      <c r="I43">
+        <v>2020</v>
+      </c>
+      <c r="J43">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>250</v>
+      </c>
+      <c r="B44" t="s">
+        <v>251</v>
+      </c>
+      <c r="C44" t="s">
+        <v>252</v>
+      </c>
+      <c r="D44" t="s">
+        <v>265</v>
+      </c>
+      <c r="E44" t="s">
+        <v>266</v>
+      </c>
+      <c r="F44" t="s">
+        <v>167</v>
+      </c>
+      <c r="G44" t="s">
+        <v>161</v>
+      </c>
+      <c r="H44">
+        <v>1219000</v>
+      </c>
+      <c r="I44">
+        <v>2017</v>
+      </c>
+      <c r="J44">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>250</v>
+      </c>
+      <c r="B45" t="s">
+        <v>251</v>
+      </c>
+      <c r="C45" t="s">
+        <v>252</v>
+      </c>
+      <c r="D45" t="s">
+        <v>267</v>
+      </c>
+      <c r="E45" t="s">
+        <v>268</v>
+      </c>
+      <c r="F45" t="s">
+        <v>167</v>
+      </c>
+      <c r="G45" t="s">
+        <v>161</v>
+      </c>
+      <c r="H45">
+        <v>1549000</v>
+      </c>
+      <c r="I45">
+        <v>2019</v>
+      </c>
+      <c r="J45">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>250</v>
+      </c>
+      <c r="B46" t="s">
+        <v>251</v>
+      </c>
+      <c r="C46" t="s">
+        <v>252</v>
+      </c>
+      <c r="D46" t="s">
+        <v>269</v>
+      </c>
+      <c r="E46" t="s">
+        <v>270</v>
+      </c>
+      <c r="F46" t="s">
+        <v>181</v>
+      </c>
+      <c r="G46" t="s">
+        <v>161</v>
+      </c>
+      <c r="H46">
+        <v>762000</v>
+      </c>
+      <c r="I46">
+        <v>2021</v>
+      </c>
+      <c r="J46">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>271</v>
+      </c>
+      <c r="B47" t="s">
+        <v>272</v>
+      </c>
+      <c r="C47" t="s">
+        <v>273</v>
+      </c>
+      <c r="D47" t="s">
+        <v>274</v>
+      </c>
+      <c r="E47" t="s">
+        <v>275</v>
+      </c>
+      <c r="F47" t="s">
+        <v>181</v>
+      </c>
+      <c r="G47" t="s">
+        <v>161</v>
+      </c>
+      <c r="H47">
+        <v>779000</v>
+      </c>
+      <c r="I47">
+        <v>2022</v>
+      </c>
+      <c r="J47">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>271</v>
+      </c>
+      <c r="B48" t="s">
+        <v>272</v>
+      </c>
+      <c r="C48" t="s">
+        <v>273</v>
+      </c>
+      <c r="D48" t="s">
+        <v>276</v>
+      </c>
+      <c r="E48" t="s">
+        <v>277</v>
+      </c>
+      <c r="F48" t="s">
+        <v>181</v>
+      </c>
+      <c r="G48" t="s">
+        <v>161</v>
+      </c>
+      <c r="H48">
+        <v>1814000</v>
+      </c>
+      <c r="I48">
+        <v>2022</v>
+      </c>
+      <c r="J48">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>271</v>
+      </c>
+      <c r="B49" t="s">
+        <v>272</v>
+      </c>
+      <c r="C49" t="s">
+        <v>273</v>
+      </c>
+      <c r="D49" t="s">
+        <v>278</v>
+      </c>
+      <c r="E49" t="s">
+        <v>279</v>
+      </c>
+      <c r="F49" t="s">
+        <v>167</v>
+      </c>
+      <c r="G49" t="s">
+        <v>161</v>
+      </c>
+      <c r="H49">
+        <v>1379000</v>
+      </c>
+      <c r="I49">
+        <v>2022</v>
+      </c>
+      <c r="J49">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>280</v>
+      </c>
+      <c r="B50" t="s">
+        <v>281</v>
+      </c>
+      <c r="C50" t="s">
+        <v>282</v>
+      </c>
+      <c r="D50" t="s">
+        <v>283</v>
+      </c>
+      <c r="E50" t="s">
+        <v>284</v>
+      </c>
+      <c r="F50" t="s">
+        <v>164</v>
+      </c>
+      <c r="G50" t="s">
+        <v>168</v>
+      </c>
+      <c r="H50">
+        <v>579900</v>
+      </c>
+      <c r="I50">
+        <v>2024</v>
+      </c>
+      <c r="J50">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>280</v>
+      </c>
+      <c r="B51" t="s">
+        <v>281</v>
+      </c>
+      <c r="C51" t="s">
+        <v>282</v>
+      </c>
+      <c r="D51" t="s">
+        <v>285</v>
+      </c>
+      <c r="E51" t="s">
+        <v>286</v>
+      </c>
+      <c r="F51" t="s">
+        <v>160</v>
+      </c>
+      <c r="G51" t="s">
+        <v>161</v>
+      </c>
+      <c r="H51">
+        <v>629900</v>
+      </c>
+      <c r="I51">
+        <v>2021</v>
+      </c>
+      <c r="J51">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>280</v>
+      </c>
+      <c r="B52" t="s">
+        <v>281</v>
+      </c>
+      <c r="C52" t="s">
+        <v>282</v>
+      </c>
+      <c r="D52" t="s">
+        <v>287</v>
+      </c>
+      <c r="E52" t="s">
+        <v>288</v>
+      </c>
+      <c r="F52" t="s">
+        <v>167</v>
+      </c>
+      <c r="G52" t="s">
+        <v>161</v>
+      </c>
+      <c r="H52">
+        <v>599000</v>
+      </c>
+      <c r="I52">
+        <v>2017</v>
+      </c>
+      <c r="J52">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>280</v>
+      </c>
+      <c r="B53" t="s">
+        <v>281</v>
+      </c>
+      <c r="C53" t="s">
+        <v>282</v>
+      </c>
+      <c r="D53" t="s">
+        <v>289</v>
+      </c>
+      <c r="E53" t="s">
+        <v>290</v>
+      </c>
+      <c r="F53" t="s">
+        <v>167</v>
+      </c>
+      <c r="G53" t="s">
+        <v>191</v>
+      </c>
+      <c r="H53">
+        <v>829900</v>
+      </c>
+      <c r="I53">
+        <v>2019</v>
+      </c>
+      <c r="J53">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>280</v>
+      </c>
+      <c r="B54" t="s">
+        <v>281</v>
+      </c>
+      <c r="C54" t="s">
+        <v>282</v>
+      </c>
+      <c r="D54" t="s">
+        <v>291</v>
+      </c>
+      <c r="E54" t="s">
+        <v>292</v>
+      </c>
+      <c r="F54" t="s">
+        <v>167</v>
+      </c>
+      <c r="G54" t="s">
+        <v>168</v>
+      </c>
+      <c r="H54">
+        <v>699000</v>
+      </c>
+      <c r="I54">
+        <v>2022</v>
+      </c>
+      <c r="J54">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>280</v>
+      </c>
+      <c r="B55" t="s">
+        <v>281</v>
+      </c>
+      <c r="C55" t="s">
+        <v>282</v>
+      </c>
+      <c r="D55" t="s">
+        <v>293</v>
+      </c>
+      <c r="E55" t="s">
+        <v>294</v>
+      </c>
+      <c r="F55" t="s">
+        <v>167</v>
+      </c>
+      <c r="G55" t="s">
+        <v>295</v>
+      </c>
+      <c r="H55">
+        <v>939000</v>
+      </c>
+      <c r="I55">
+        <v>2020</v>
+      </c>
+      <c r="J55">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>280</v>
+      </c>
+      <c r="B56" t="s">
+        <v>281</v>
+      </c>
+      <c r="C56" t="s">
+        <v>282</v>
+      </c>
+      <c r="D56" t="s">
+        <v>296</v>
+      </c>
+      <c r="E56" t="s">
+        <v>297</v>
+      </c>
+      <c r="F56" t="s">
+        <v>164</v>
+      </c>
+      <c r="G56" t="s">
+        <v>191</v>
+      </c>
+      <c r="H56">
+        <v>669900</v>
+      </c>
+      <c r="I56">
+        <v>2022</v>
+      </c>
+      <c r="J56">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>280</v>
+      </c>
+      <c r="B57" t="s">
+        <v>281</v>
+      </c>
+      <c r="C57" t="s">
+        <v>282</v>
+      </c>
+      <c r="D57" t="s">
+        <v>298</v>
+      </c>
+      <c r="E57" t="s">
+        <v>299</v>
+      </c>
+      <c r="F57" t="s">
+        <v>164</v>
+      </c>
+      <c r="G57" t="s">
+        <v>191</v>
+      </c>
+      <c r="H57">
+        <v>771000</v>
+      </c>
+      <c r="I57">
+        <v>2020</v>
+      </c>
+      <c r="J57">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>280</v>
+      </c>
+      <c r="B58" t="s">
+        <v>281</v>
+      </c>
+      <c r="C58" t="s">
+        <v>282</v>
+      </c>
+      <c r="D58" t="s">
+        <v>300</v>
+      </c>
+      <c r="E58" t="s">
+        <v>301</v>
+      </c>
+      <c r="F58" t="s">
+        <v>164</v>
+      </c>
+      <c r="G58" t="s">
+        <v>191</v>
+      </c>
+      <c r="H58">
+        <v>959000</v>
+      </c>
+      <c r="I58">
+        <v>2023</v>
+      </c>
+      <c r="J58">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>280</v>
+      </c>
+      <c r="B59" t="s">
+        <v>281</v>
+      </c>
+      <c r="C59" t="s">
+        <v>282</v>
+      </c>
+      <c r="D59" t="s">
+        <v>302</v>
+      </c>
+      <c r="E59" t="s">
+        <v>303</v>
+      </c>
+      <c r="F59" t="s">
+        <v>186</v>
+      </c>
+      <c r="G59" t="s">
+        <v>191</v>
+      </c>
+      <c r="H59">
+        <v>1399000</v>
+      </c>
+      <c r="I59">
+        <v>2024</v>
+      </c>
+      <c r="J59">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>280</v>
+      </c>
+      <c r="B60" t="s">
+        <v>281</v>
+      </c>
+      <c r="C60" t="s">
+        <v>282</v>
+      </c>
+      <c r="D60" t="s">
+        <v>304</v>
+      </c>
+      <c r="E60" t="s">
+        <v>305</v>
+      </c>
+      <c r="F60" t="s">
+        <v>186</v>
+      </c>
+      <c r="G60" t="s">
+        <v>191</v>
+      </c>
+      <c r="H60">
+        <v>1849900</v>
+      </c>
+      <c r="I60">
+        <v>2023</v>
+      </c>
+      <c r="J60">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>280</v>
+      </c>
+      <c r="B61" t="s">
+        <v>281</v>
+      </c>
+      <c r="C61" t="s">
+        <v>282</v>
+      </c>
+      <c r="D61" t="s">
+        <v>306</v>
+      </c>
+      <c r="E61" t="s">
+        <v>307</v>
+      </c>
+      <c r="F61" t="s">
+        <v>181</v>
+      </c>
+      <c r="G61" t="s">
+        <v>161</v>
+      </c>
+      <c r="H61">
+        <v>589000</v>
+      </c>
+      <c r="I61">
+        <v>2019</v>
+      </c>
+      <c r="J61">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>308</v>
+      </c>
+      <c r="B62" t="s">
+        <v>309</v>
+      </c>
+      <c r="C62" t="s">
+        <v>310</v>
+      </c>
+      <c r="D62" t="s">
+        <v>311</v>
+      </c>
+      <c r="E62" t="s">
+        <v>312</v>
+      </c>
+      <c r="F62" t="s">
+        <v>164</v>
+      </c>
+      <c r="G62" t="s">
+        <v>191</v>
+      </c>
+      <c r="H62">
+        <v>499900</v>
+      </c>
+      <c r="I62">
+        <v>2023</v>
+      </c>
+      <c r="J62">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>308</v>
+      </c>
+      <c r="B63" t="s">
+        <v>309</v>
+      </c>
+      <c r="C63" t="s">
+        <v>310</v>
+      </c>
+      <c r="D63" t="s">
+        <v>313</v>
+      </c>
+      <c r="E63" t="s">
+        <v>314</v>
+      </c>
+      <c r="F63" t="s">
+        <v>167</v>
+      </c>
+      <c r="G63" t="s">
+        <v>191</v>
+      </c>
+      <c r="H63">
+        <v>669900</v>
+      </c>
+      <c r="I63">
+        <v>2022</v>
+      </c>
+      <c r="J63">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>308</v>
+      </c>
+      <c r="B64" t="s">
+        <v>309</v>
+      </c>
+      <c r="C64" t="s">
+        <v>310</v>
+      </c>
+      <c r="D64" t="s">
+        <v>315</v>
+      </c>
+      <c r="E64" t="s">
+        <v>316</v>
+      </c>
+      <c r="F64" t="s">
+        <v>160</v>
+      </c>
+      <c r="G64" t="s">
+        <v>191</v>
+      </c>
+      <c r="H64">
+        <v>999900</v>
+      </c>
+      <c r="I64">
+        <v>2023</v>
+      </c>
+      <c r="J64">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>308</v>
+      </c>
+      <c r="B65" t="s">
+        <v>309</v>
+      </c>
+      <c r="C65" t="s">
+        <v>310</v>
+      </c>
+      <c r="D65" t="s">
+        <v>317</v>
+      </c>
+      <c r="E65" t="s">
+        <v>318</v>
+      </c>
+      <c r="F65" t="s">
+        <v>167</v>
+      </c>
+      <c r="G65" t="s">
+        <v>295</v>
+      </c>
+      <c r="H65">
+        <v>699900</v>
+      </c>
+      <c r="I65">
+        <v>2024</v>
+      </c>
+      <c r="J65">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>308</v>
+      </c>
+      <c r="B66" t="s">
+        <v>309</v>
+      </c>
+      <c r="C66" t="s">
+        <v>310</v>
+      </c>
+      <c r="D66" t="s">
+        <v>319</v>
+      </c>
+      <c r="E66" t="s">
+        <v>320</v>
+      </c>
+      <c r="F66" t="s">
+        <v>186</v>
+      </c>
+      <c r="G66" t="s">
+        <v>191</v>
+      </c>
+      <c r="H66">
+        <v>799900</v>
+      </c>
+      <c r="I66">
+        <v>2024</v>
+      </c>
+      <c r="J66">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>308</v>
+      </c>
+      <c r="B67" t="s">
+        <v>309</v>
+      </c>
+      <c r="C67" t="s">
+        <v>310</v>
+      </c>
+      <c r="D67" t="s">
+        <v>321</v>
+      </c>
+      <c r="E67" t="s">
+        <v>322</v>
+      </c>
+      <c r="F67" t="s">
+        <v>167</v>
+      </c>
+      <c r="G67" t="s">
+        <v>191</v>
+      </c>
+      <c r="H67">
+        <v>1149900</v>
+      </c>
+      <c r="I67">
+        <v>2024</v>
+      </c>
+      <c r="J67">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>323</v>
+      </c>
+      <c r="B68" t="s">
+        <v>324</v>
+      </c>
+      <c r="C68" t="s">
+        <v>325</v>
+      </c>
+      <c r="D68" t="s">
+        <v>326</v>
+      </c>
+      <c r="E68" t="s">
+        <v>327</v>
+      </c>
+      <c r="F68" t="s">
+        <v>164</v>
+      </c>
+      <c r="G68" t="s">
+        <v>161</v>
+      </c>
+      <c r="H68">
+        <v>319900</v>
+      </c>
+      <c r="I68">
+        <v>2015</v>
+      </c>
+      <c r="J68">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>323</v>
+      </c>
+      <c r="B69" t="s">
+        <v>324</v>
+      </c>
+      <c r="C69" t="s">
+        <v>325</v>
+      </c>
+      <c r="D69" t="s">
+        <v>328</v>
+      </c>
+      <c r="E69" t="s">
+        <v>329</v>
+      </c>
+      <c r="F69" t="s">
+        <v>164</v>
+      </c>
+      <c r="G69" t="s">
+        <v>161</v>
+      </c>
+      <c r="H69">
+        <v>567000</v>
+      </c>
+      <c r="I69">
+        <v>2018</v>
+      </c>
+      <c r="J69">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>323</v>
+      </c>
+      <c r="B70" t="s">
+        <v>324</v>
+      </c>
+      <c r="C70" t="s">
+        <v>325</v>
+      </c>
+      <c r="D70" t="s">
+        <v>330</v>
+      </c>
+      <c r="E70" t="s">
+        <v>331</v>
+      </c>
+      <c r="F70" t="s">
+        <v>186</v>
+      </c>
+      <c r="G70" t="s">
+        <v>168</v>
+      </c>
+      <c r="H70">
+        <v>799000</v>
+      </c>
+      <c r="I70">
+        <v>2024</v>
+      </c>
+      <c r="J70">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>323</v>
+      </c>
+      <c r="B71" t="s">
+        <v>324</v>
+      </c>
+      <c r="C71" t="s">
+        <v>325</v>
+      </c>
+      <c r="D71" t="s">
+        <v>332</v>
+      </c>
+      <c r="E71" t="s">
+        <v>333</v>
+      </c>
+      <c r="F71" t="s">
+        <v>181</v>
+      </c>
+      <c r="G71" t="s">
+        <v>161</v>
+      </c>
+      <c r="H71">
+        <v>395000</v>
+      </c>
+      <c r="I71">
+        <v>2019</v>
+      </c>
+      <c r="J71">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>323</v>
+      </c>
+      <c r="B72" t="s">
+        <v>324</v>
+      </c>
+      <c r="C72" t="s">
+        <v>325</v>
+      </c>
+      <c r="D72" t="s">
+        <v>334</v>
+      </c>
+      <c r="E72" t="s">
+        <v>335</v>
+      </c>
+      <c r="F72" t="s">
+        <v>167</v>
+      </c>
+      <c r="G72" t="s">
+        <v>161</v>
+      </c>
+      <c r="H72">
+        <v>1450000</v>
+      </c>
+      <c r="I72">
+        <v>2019</v>
+      </c>
+      <c r="J72">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>336</v>
+      </c>
+      <c r="B73" t="s">
+        <v>337</v>
+      </c>
+      <c r="C73" t="s">
+        <v>338</v>
+      </c>
+      <c r="D73" t="s">
+        <v>339</v>
+      </c>
+      <c r="E73" t="s">
+        <v>340</v>
+      </c>
+      <c r="F73" t="s">
+        <v>167</v>
+      </c>
+      <c r="G73" t="s">
+        <v>168</v>
+      </c>
+      <c r="H73">
+        <v>899000</v>
+      </c>
+      <c r="I73">
+        <v>2021</v>
+      </c>
+      <c r="J73">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>336</v>
+      </c>
+      <c r="B74" t="s">
+        <v>337</v>
+      </c>
+      <c r="C74" t="s">
+        <v>338</v>
+      </c>
+      <c r="D74" t="s">
+        <v>341</v>
+      </c>
+      <c r="E74" t="s">
+        <v>342</v>
+      </c>
+      <c r="F74" t="s">
+        <v>167</v>
+      </c>
+      <c r="G74" t="s">
+        <v>295</v>
+      </c>
+      <c r="H74">
+        <v>959000</v>
+      </c>
+      <c r="I74">
+        <v>2022</v>
+      </c>
+      <c r="J74">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>336</v>
+      </c>
+      <c r="B75" t="s">
+        <v>337</v>
+      </c>
+      <c r="C75" t="s">
+        <v>338</v>
+      </c>
+      <c r="D75" t="s">
+        <v>343</v>
+      </c>
+      <c r="E75" t="s">
+        <v>344</v>
+      </c>
+      <c r="F75" t="s">
+        <v>164</v>
+      </c>
+      <c r="G75" t="s">
+        <v>191</v>
+      </c>
+      <c r="H75">
+        <v>799000</v>
+      </c>
+      <c r="I75">
+        <v>2021</v>
+      </c>
+      <c r="J75">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>336</v>
+      </c>
+      <c r="B76" t="s">
+        <v>337</v>
+      </c>
+      <c r="C76" t="s">
+        <v>338</v>
+      </c>
+      <c r="D76" t="s">
+        <v>345</v>
+      </c>
+      <c r="E76" t="s">
+        <v>346</v>
+      </c>
+      <c r="F76" t="s">
+        <v>160</v>
+      </c>
+      <c r="G76" t="s">
+        <v>191</v>
+      </c>
+      <c r="H76">
+        <v>1299000</v>
+      </c>
+      <c r="I76">
+        <v>2023</v>
+      </c>
+      <c r="J76">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>336</v>
+      </c>
+      <c r="B77" t="s">
+        <v>337</v>
+      </c>
+      <c r="C77" t="s">
+        <v>338</v>
+      </c>
+      <c r="D77" t="s">
+        <v>347</v>
+      </c>
+      <c r="E77" t="s">
+        <v>348</v>
+      </c>
+      <c r="F77" t="s">
+        <v>167</v>
+      </c>
+      <c r="G77" t="s">
+        <v>191</v>
+      </c>
+      <c r="H77">
+        <v>649000</v>
+      </c>
+      <c r="I77">
+        <v>2025</v>
+      </c>
+      <c r="J77">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>336</v>
+      </c>
+      <c r="B78" t="s">
+        <v>337</v>
+      </c>
+      <c r="C78" t="s">
+        <v>338</v>
+      </c>
+      <c r="D78" t="s">
+        <v>349</v>
+      </c>
+      <c r="E78" t="s">
+        <v>350</v>
+      </c>
+      <c r="F78" t="s">
+        <v>167</v>
+      </c>
+      <c r="G78" t="s">
+        <v>168</v>
+      </c>
+      <c r="H78">
+        <v>709000</v>
+      </c>
+      <c r="I78">
+        <v>2025</v>
+      </c>
+      <c r="J78">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>336</v>
+      </c>
+      <c r="B79" t="s">
+        <v>337</v>
+      </c>
+      <c r="C79" t="s">
+        <v>338</v>
+      </c>
+      <c r="D79" t="s">
+        <v>351</v>
+      </c>
+      <c r="E79" t="s">
+        <v>352</v>
+      </c>
+      <c r="F79" t="s">
+        <v>167</v>
+      </c>
+      <c r="G79" t="s">
+        <v>168</v>
+      </c>
+      <c r="H79">
+        <v>1649000</v>
+      </c>
+      <c r="I79">
+        <v>2023</v>
+      </c>
+      <c r="J79">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>336</v>
+      </c>
+      <c r="B80" t="s">
+        <v>337</v>
+      </c>
+      <c r="C80" t="s">
+        <v>338</v>
+      </c>
+      <c r="D80" t="s">
+        <v>353</v>
+      </c>
+      <c r="E80" t="s">
+        <v>354</v>
+      </c>
+      <c r="F80" t="s">
+        <v>167</v>
+      </c>
+      <c r="G80" t="s">
+        <v>168</v>
+      </c>
+      <c r="H80">
+        <v>2049000</v>
+      </c>
+      <c r="I80">
+        <v>2023</v>
+      </c>
+      <c r="J80">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>336</v>
+      </c>
+      <c r="B81" t="s">
+        <v>337</v>
+      </c>
+      <c r="C81" t="s">
+        <v>338</v>
+      </c>
+      <c r="D81" t="s">
+        <v>355</v>
+      </c>
+      <c r="E81" t="s">
+        <v>356</v>
+      </c>
+      <c r="F81" t="s">
+        <v>181</v>
+      </c>
+      <c r="G81" t="s">
+        <v>168</v>
+      </c>
+      <c r="H81">
+        <v>1189000</v>
+      </c>
+      <c r="I81">
+        <v>2024</v>
+      </c>
+      <c r="J81">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>357</v>
+      </c>
+      <c r="B82" t="s">
+        <v>358</v>
+      </c>
+      <c r="C82" t="s">
+        <v>359</v>
+      </c>
+      <c r="D82" t="s">
+        <v>360</v>
+      </c>
+      <c r="E82" t="s">
+        <v>361</v>
+      </c>
+      <c r="F82" t="s">
+        <v>167</v>
+      </c>
+      <c r="G82" t="s">
+        <v>161</v>
+      </c>
+      <c r="H82">
+        <v>929000</v>
+      </c>
+      <c r="I82">
+        <v>2022</v>
+      </c>
+      <c r="J82">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>357</v>
+      </c>
+      <c r="B83" t="s">
+        <v>358</v>
+      </c>
+      <c r="C83" t="s">
+        <v>359</v>
+      </c>
+      <c r="D83" t="s">
+        <v>362</v>
+      </c>
+      <c r="E83" t="s">
+        <v>363</v>
+      </c>
+      <c r="F83" t="s">
+        <v>186</v>
+      </c>
+      <c r="G83" t="s">
+        <v>161</v>
+      </c>
+      <c r="H83">
+        <v>795000</v>
+      </c>
+      <c r="I83">
+        <v>2023</v>
+      </c>
+      <c r="J83">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>357</v>
+      </c>
+      <c r="B84" t="s">
+        <v>358</v>
+      </c>
+      <c r="C84" t="s">
+        <v>359</v>
+      </c>
+      <c r="D84" t="s">
+        <v>364</v>
+      </c>
+      <c r="E84" t="s">
+        <v>365</v>
+      </c>
+      <c r="F84" t="s">
+        <v>186</v>
+      </c>
+      <c r="G84" t="s">
+        <v>161</v>
+      </c>
+      <c r="H84">
+        <v>1659000</v>
+      </c>
+      <c r="I84">
+        <v>2021</v>
+      </c>
+      <c r="J84">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>357</v>
+      </c>
+      <c r="B85" t="s">
+        <v>358</v>
+      </c>
+      <c r="C85" t="s">
+        <v>359</v>
+      </c>
+      <c r="D85" t="s">
+        <v>366</v>
+      </c>
+      <c r="E85" t="s">
+        <v>367</v>
+      </c>
+      <c r="F85" t="s">
+        <v>186</v>
+      </c>
+      <c r="G85" t="s">
+        <v>168</v>
+      </c>
+      <c r="H85">
+        <v>2099000</v>
+      </c>
+      <c r="I85">
+        <v>2025</v>
+      </c>
+      <c r="J85">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>357</v>
+      </c>
+      <c r="B86" t="s">
+        <v>358</v>
+      </c>
+      <c r="C86" t="s">
+        <v>359</v>
+      </c>
+      <c r="D86" t="s">
+        <v>368</v>
+      </c>
+      <c r="E86" t="s">
+        <v>369</v>
+      </c>
+      <c r="F86" t="s">
+        <v>167</v>
+      </c>
+      <c r="G86" t="s">
+        <v>168</v>
+      </c>
+      <c r="H86">
+        <v>1599000</v>
+      </c>
+      <c r="I86">
+        <v>2023</v>
+      </c>
+      <c r="J86">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>357</v>
+      </c>
+      <c r="B87" t="s">
+        <v>358</v>
+      </c>
+      <c r="C87" t="s">
+        <v>359</v>
+      </c>
+      <c r="D87" t="s">
+        <v>370</v>
+      </c>
+      <c r="E87" t="s">
+        <v>371</v>
+      </c>
+      <c r="F87" t="s">
+        <v>167</v>
+      </c>
+      <c r="G87" t="s">
+        <v>191</v>
+      </c>
+      <c r="H87">
+        <v>1699000</v>
+      </c>
+      <c r="I87">
+        <v>2023</v>
+      </c>
+      <c r="J87">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>357</v>
+      </c>
+      <c r="B88" t="s">
+        <v>358</v>
+      </c>
+      <c r="C88" t="s">
+        <v>359</v>
+      </c>
+      <c r="D88" t="s">
+        <v>372</v>
+      </c>
+      <c r="E88" t="s">
+        <v>373</v>
+      </c>
+      <c r="F88" t="s">
+        <v>167</v>
+      </c>
+      <c r="G88" t="s">
+        <v>161</v>
+      </c>
+      <c r="H88">
+        <v>2299000</v>
+      </c>
+      <c r="I88">
+        <v>2024</v>
+      </c>
+      <c r="J88">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>374</v>
+      </c>
+      <c r="B89" t="s">
+        <v>375</v>
+      </c>
+      <c r="C89" t="s">
+        <v>376</v>
+      </c>
+      <c r="D89" t="s">
+        <v>377</v>
+      </c>
+      <c r="E89" t="s">
+        <v>378</v>
+      </c>
+      <c r="F89" t="s">
+        <v>160</v>
+      </c>
+      <c r="G89" t="s">
+        <v>191</v>
+      </c>
+      <c r="H89">
+        <v>1149000</v>
+      </c>
+      <c r="I89">
+        <v>2022</v>
+      </c>
+      <c r="J89">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>374</v>
+      </c>
+      <c r="B90" t="s">
+        <v>375</v>
+      </c>
+      <c r="C90" t="s">
+        <v>376</v>
+      </c>
+      <c r="D90" t="s">
+        <v>379</v>
+      </c>
+      <c r="E90" t="s">
+        <v>380</v>
+      </c>
+      <c r="F90" t="s">
+        <v>167</v>
+      </c>
+      <c r="G90" t="s">
+        <v>191</v>
+      </c>
+      <c r="H90">
+        <v>1769000</v>
+      </c>
+      <c r="I90">
+        <v>2022</v>
+      </c>
+      <c r="J90">
+        <v>2026</v>
+      </c>
+    </row>
     <row r="91" spans="6:7" x14ac:dyDescent="0.25"/>
     <row r="92" spans="6:7" x14ac:dyDescent="0.25"/>
     <row r="93" spans="6:7" x14ac:dyDescent="0.25"/>
@@ -4073,40 +6877,40 @@
         <v>143</v>
       </c>
       <c r="B2" t="s">
-        <v>211</v>
+        <v>381</v>
       </c>
       <c r="C2" t="s">
-        <v>212</v>
+        <v>382</v>
       </c>
       <c r="D2" t="s">
-        <v>213</v>
+        <v>383</v>
       </c>
       <c r="E2" t="s">
-        <v>214</v>
+        <v>384</v>
       </c>
       <c r="F2" t="s">
-        <v>215</v>
+        <v>385</v>
       </c>
       <c r="G2" t="s">
-        <v>216</v>
+        <v>386</v>
       </c>
       <c r="H2" t="s">
-        <v>217</v>
+        <v>387</v>
       </c>
       <c r="I2">
         <v>0</v>
       </c>
       <c r="J2" t="s">
-        <v>218</v>
+        <v>388</v>
       </c>
       <c r="K2" t="s">
-        <v>218</v>
+        <v>388</v>
       </c>
       <c r="L2" t="s">
-        <v>218</v>
+        <v>388</v>
       </c>
       <c r="M2" t="s">
-        <v>218</v>
+        <v>388</v>
       </c>
       <c r="N2">
         <v>1000000</v>
@@ -4130,16 +6934,16 @@
         <v>5</v>
       </c>
       <c r="U2" t="s">
-        <v>218</v>
+        <v>388</v>
       </c>
       <c r="V2">
         <v>0</v>
       </c>
       <c r="W2" t="s">
-        <v>219</v>
+        <v>389</v>
       </c>
       <c r="X2" t="s">
-        <v>219</v>
+        <v>389</v>
       </c>
       <c r="Y2" t="s">
         <v>105</v>
@@ -4157,16 +6961,16 @@
         <v>5</v>
       </c>
       <c r="AM2" t="s">
-        <v>220</v>
+        <v>390</v>
       </c>
       <c r="AN2" t="s">
-        <v>221</v>
+        <v>391</v>
       </c>
       <c r="AO2" t="s">
-        <v>222</v>
+        <v>392</v>
       </c>
       <c r="AQ2" t="s">
-        <v>223</v>
+        <v>393</v>
       </c>
     </row>
     <row r="3" spans="1:43" x14ac:dyDescent="0.25">
@@ -4174,40 +6978,40 @@
         <v>143</v>
       </c>
       <c r="B3" t="s">
-        <v>211</v>
+        <v>381</v>
       </c>
       <c r="C3" t="s">
-        <v>212</v>
+        <v>382</v>
       </c>
       <c r="D3" t="s">
-        <v>213</v>
+        <v>383</v>
       </c>
       <c r="E3" t="s">
-        <v>214</v>
+        <v>384</v>
       </c>
       <c r="F3" t="s">
-        <v>224</v>
+        <v>394</v>
       </c>
       <c r="G3" t="s">
-        <v>225</v>
+        <v>395</v>
       </c>
       <c r="H3" t="s">
-        <v>217</v>
+        <v>387</v>
       </c>
       <c r="I3">
         <v>0</v>
       </c>
       <c r="J3" t="s">
-        <v>218</v>
+        <v>388</v>
       </c>
       <c r="K3" t="s">
-        <v>218</v>
+        <v>388</v>
       </c>
       <c r="L3" t="s">
-        <v>218</v>
+        <v>388</v>
       </c>
       <c r="M3" t="s">
-        <v>218</v>
+        <v>388</v>
       </c>
       <c r="N3">
         <v>1000000</v>
@@ -4231,16 +7035,16 @@
         <v>5</v>
       </c>
       <c r="U3" t="s">
-        <v>218</v>
+        <v>388</v>
       </c>
       <c r="V3">
         <v>0</v>
       </c>
       <c r="W3" t="s">
-        <v>219</v>
+        <v>389</v>
       </c>
       <c r="X3" t="s">
-        <v>219</v>
+        <v>389</v>
       </c>
       <c r="Y3" t="s">
         <v>105</v>
@@ -4258,16 +7062,16 @@
         <v>5</v>
       </c>
       <c r="AM3" t="s">
-        <v>226</v>
+        <v>396</v>
       </c>
       <c r="AN3" t="s">
-        <v>227</v>
+        <v>397</v>
       </c>
       <c r="AO3" t="s">
-        <v>222</v>
+        <v>392</v>
       </c>
       <c r="AQ3" t="s">
-        <v>223</v>
+        <v>393</v>
       </c>
     </row>
     <row r="4" spans="1:43" x14ac:dyDescent="0.25">
@@ -4275,40 +7079,40 @@
         <v>147</v>
       </c>
       <c r="B4" t="s">
-        <v>228</v>
+        <v>398</v>
       </c>
       <c r="C4" t="s">
-        <v>229</v>
+        <v>399</v>
       </c>
       <c r="D4" t="s">
-        <v>230</v>
+        <v>400</v>
       </c>
       <c r="E4" t="s">
-        <v>214</v>
+        <v>384</v>
       </c>
       <c r="F4" t="s">
-        <v>215</v>
+        <v>385</v>
       </c>
       <c r="G4" t="s">
-        <v>225</v>
+        <v>395</v>
       </c>
       <c r="H4" t="s">
-        <v>231</v>
+        <v>401</v>
       </c>
       <c r="I4">
         <v>2000</v>
       </c>
       <c r="J4" t="s">
-        <v>218</v>
+        <v>388</v>
       </c>
       <c r="K4" t="s">
-        <v>218</v>
+        <v>388</v>
       </c>
       <c r="L4" t="s">
-        <v>218</v>
+        <v>388</v>
       </c>
       <c r="M4" t="s">
-        <v>218</v>
+        <v>388</v>
       </c>
       <c r="N4">
         <v>1000000</v>
@@ -4332,16 +7136,16 @@
         <v>5</v>
       </c>
       <c r="U4" t="s">
-        <v>218</v>
+        <v>388</v>
       </c>
       <c r="V4">
         <v>0</v>
       </c>
       <c r="W4" t="s">
-        <v>219</v>
+        <v>389</v>
       </c>
       <c r="X4" t="s">
-        <v>219</v>
+        <v>389</v>
       </c>
       <c r="Y4" t="s">
         <v>105</v>
@@ -4359,16 +7163,16 @@
         <v>12</v>
       </c>
       <c r="AM4" t="s">
-        <v>220</v>
+        <v>390</v>
       </c>
       <c r="AN4" t="s">
-        <v>232</v>
+        <v>402</v>
       </c>
       <c r="AO4" t="s">
-        <v>222</v>
+        <v>392</v>
       </c>
       <c r="AQ4" t="s">
-        <v>223</v>
+        <v>393</v>
       </c>
     </row>
     <row r="5" spans="1:43" x14ac:dyDescent="0.25">
@@ -4376,40 +7180,40 @@
         <v>151</v>
       </c>
       <c r="B5" t="s">
-        <v>233</v>
+        <v>403</v>
       </c>
       <c r="C5" t="s">
-        <v>234</v>
+        <v>404</v>
       </c>
       <c r="D5" t="s">
-        <v>235</v>
+        <v>405</v>
       </c>
       <c r="E5" t="s">
-        <v>214</v>
+        <v>384</v>
       </c>
       <c r="F5" t="s">
-        <v>215</v>
+        <v>385</v>
       </c>
       <c r="G5" t="s">
-        <v>225</v>
+        <v>395</v>
       </c>
       <c r="H5" t="s">
-        <v>217</v>
+        <v>387</v>
       </c>
       <c r="I5">
         <v>0</v>
       </c>
       <c r="J5" t="s">
-        <v>218</v>
+        <v>388</v>
       </c>
       <c r="K5" t="s">
-        <v>218</v>
+        <v>388</v>
       </c>
       <c r="L5" t="s">
-        <v>218</v>
+        <v>388</v>
       </c>
       <c r="M5" t="s">
-        <v>218</v>
+        <v>388</v>
       </c>
       <c r="N5">
         <v>1000000</v>
@@ -4433,16 +7237,16 @@
         <v>5</v>
       </c>
       <c r="U5" t="s">
-        <v>218</v>
+        <v>388</v>
       </c>
       <c r="V5">
         <v>7</v>
       </c>
       <c r="W5" t="s">
-        <v>219</v>
+        <v>389</v>
       </c>
       <c r="X5" t="s">
-        <v>219</v>
+        <v>389</v>
       </c>
       <c r="Y5" t="s">
         <v>105</v>
@@ -4460,16 +7264,16 @@
         <v>7</v>
       </c>
       <c r="AM5" t="s">
-        <v>236</v>
+        <v>406</v>
       </c>
       <c r="AN5" t="s">
-        <v>237</v>
+        <v>407</v>
       </c>
       <c r="AO5" t="s">
-        <v>222</v>
+        <v>392</v>
       </c>
       <c r="AQ5" t="s">
-        <v>223</v>
+        <v>393</v>
       </c>
     </row>
     <row r="6" spans="1:43" x14ac:dyDescent="0.25">
@@ -4477,40 +7281,40 @@
         <v>151</v>
       </c>
       <c r="B6" t="s">
-        <v>238</v>
+        <v>408</v>
       </c>
       <c r="C6" t="s">
-        <v>239</v>
+        <v>409</v>
       </c>
       <c r="D6" t="s">
-        <v>240</v>
+        <v>410</v>
       </c>
       <c r="E6" t="s">
-        <v>214</v>
+        <v>384</v>
       </c>
       <c r="F6" t="s">
-        <v>215</v>
+        <v>385</v>
       </c>
       <c r="G6" t="s">
-        <v>225</v>
+        <v>395</v>
       </c>
       <c r="H6" t="s">
-        <v>231</v>
+        <v>401</v>
       </c>
       <c r="I6">
         <v>0</v>
       </c>
       <c r="J6" t="s">
-        <v>218</v>
+        <v>388</v>
       </c>
       <c r="K6" t="s">
-        <v>218</v>
+        <v>388</v>
       </c>
       <c r="L6" t="s">
-        <v>218</v>
+        <v>388</v>
       </c>
       <c r="M6" t="s">
-        <v>219</v>
+        <v>389</v>
       </c>
       <c r="N6">
         <v>1000000</v>
@@ -4534,16 +7338,16 @@
         <v>5</v>
       </c>
       <c r="U6" t="s">
-        <v>219</v>
+        <v>389</v>
       </c>
       <c r="V6">
         <v>0</v>
       </c>
       <c r="W6" t="s">
-        <v>219</v>
+        <v>389</v>
       </c>
       <c r="X6" t="s">
-        <v>219</v>
+        <v>389</v>
       </c>
       <c r="Y6" t="s">
         <v>105</v>
@@ -4561,13 +7365,13 @@
         <v>15</v>
       </c>
       <c r="AN6" t="s">
-        <v>241</v>
+        <v>411</v>
       </c>
       <c r="AO6" t="s">
-        <v>222</v>
+        <v>392</v>
       </c>
       <c r="AQ6" t="s">
-        <v>223</v>
+        <v>393</v>
       </c>
     </row>
     <row r="7" spans="1:43" x14ac:dyDescent="0.25">
@@ -4575,40 +7379,40 @@
         <v>151</v>
       </c>
       <c r="B7" t="s">
-        <v>242</v>
+        <v>412</v>
       </c>
       <c r="C7" t="s">
-        <v>243</v>
+        <v>413</v>
       </c>
       <c r="D7" t="s">
-        <v>244</v>
+        <v>414</v>
       </c>
       <c r="E7" t="s">
-        <v>214</v>
+        <v>384</v>
       </c>
       <c r="F7" t="s">
-        <v>215</v>
+        <v>385</v>
       </c>
       <c r="G7" t="s">
-        <v>225</v>
+        <v>395</v>
       </c>
       <c r="H7" t="s">
-        <v>217</v>
+        <v>387</v>
       </c>
       <c r="I7">
         <v>0</v>
       </c>
       <c r="J7" t="s">
-        <v>218</v>
+        <v>388</v>
       </c>
       <c r="K7" t="s">
-        <v>218</v>
+        <v>388</v>
       </c>
       <c r="L7" t="s">
-        <v>218</v>
+        <v>388</v>
       </c>
       <c r="M7" t="s">
-        <v>218</v>
+        <v>388</v>
       </c>
       <c r="N7">
         <v>1000000</v>
@@ -4632,16 +7436,16 @@
         <v>5</v>
       </c>
       <c r="U7" t="s">
-        <v>218</v>
+        <v>388</v>
       </c>
       <c r="V7">
         <v>5</v>
       </c>
       <c r="W7" t="s">
-        <v>218</v>
+        <v>388</v>
       </c>
       <c r="X7" t="s">
-        <v>218</v>
+        <v>388</v>
       </c>
       <c r="Y7" t="s">
         <v>105</v>
@@ -4659,19 +7463,19 @@
         <v>5</v>
       </c>
       <c r="AK7" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="AM7" t="s">
-        <v>245</v>
+        <v>415</v>
       </c>
       <c r="AN7" t="s">
-        <v>246</v>
+        <v>416</v>
       </c>
       <c r="AO7" t="s">
-        <v>222</v>
+        <v>392</v>
       </c>
       <c r="AQ7" t="s">
-        <v>223</v>
+        <v>393</v>
       </c>
     </row>
     <row r="8" spans="1:43" x14ac:dyDescent="0.25">
@@ -4679,40 +7483,40 @@
         <v>143</v>
       </c>
       <c r="B8" t="s">
-        <v>247</v>
+        <v>417</v>
       </c>
       <c r="C8" t="s">
-        <v>248</v>
+        <v>418</v>
       </c>
       <c r="D8" t="s">
-        <v>249</v>
+        <v>419</v>
       </c>
       <c r="E8" t="s">
-        <v>250</v>
+        <v>420</v>
       </c>
       <c r="F8" t="s">
-        <v>215</v>
+        <v>385</v>
       </c>
       <c r="G8" t="s">
-        <v>225</v>
+        <v>395</v>
       </c>
       <c r="H8" t="s">
-        <v>231</v>
+        <v>401</v>
       </c>
       <c r="I8">
         <v>0</v>
       </c>
       <c r="J8" t="s">
-        <v>218</v>
+        <v>388</v>
       </c>
       <c r="K8" t="s">
-        <v>219</v>
+        <v>389</v>
       </c>
       <c r="L8" t="s">
-        <v>218</v>
+        <v>388</v>
       </c>
       <c r="M8" t="s">
-        <v>218</v>
+        <v>388</v>
       </c>
       <c r="N8">
         <v>1000000</v>
@@ -4736,19 +7540,19 @@
         <v>5</v>
       </c>
       <c r="U8" t="s">
-        <v>218</v>
+        <v>388</v>
       </c>
       <c r="V8">
         <v>0</v>
       </c>
       <c r="W8" t="s">
-        <v>219</v>
+        <v>389</v>
       </c>
       <c r="X8" t="s">
-        <v>219</v>
+        <v>389</v>
       </c>
       <c r="Y8" t="s">
-        <v>251</v>
+        <v>421</v>
       </c>
       <c r="AC8">
         <v>200000</v>
@@ -4769,16 +7573,16 @@
         <v>9200</v>
       </c>
       <c r="AM8" t="s">
-        <v>220</v>
+        <v>390</v>
       </c>
       <c r="AN8" t="s">
-        <v>252</v>
+        <v>422</v>
       </c>
       <c r="AO8" t="s">
-        <v>222</v>
+        <v>392</v>
       </c>
       <c r="AQ8" t="s">
-        <v>223</v>
+        <v>393</v>
       </c>
     </row>
     <row r="9" spans="1:43" x14ac:dyDescent="0.25">
@@ -4786,40 +7590,40 @@
         <v>147</v>
       </c>
       <c r="B9" t="s">
-        <v>253</v>
+        <v>423</v>
       </c>
       <c r="C9" t="s">
-        <v>254</v>
+        <v>424</v>
       </c>
       <c r="D9" t="s">
-        <v>255</v>
+        <v>425</v>
       </c>
       <c r="E9" t="s">
-        <v>256</v>
+        <v>426</v>
       </c>
       <c r="F9" t="s">
-        <v>215</v>
+        <v>385</v>
       </c>
       <c r="G9" t="s">
-        <v>225</v>
+        <v>395</v>
       </c>
       <c r="H9" t="s">
-        <v>231</v>
+        <v>401</v>
       </c>
       <c r="I9">
         <v>0</v>
       </c>
       <c r="J9" t="s">
-        <v>218</v>
+        <v>388</v>
       </c>
       <c r="K9" t="s">
-        <v>219</v>
+        <v>389</v>
       </c>
       <c r="L9" t="s">
-        <v>219</v>
+        <v>389</v>
       </c>
       <c r="M9" t="s">
-        <v>219</v>
+        <v>389</v>
       </c>
       <c r="N9">
         <v>1000000</v>
@@ -4843,19 +7647,19 @@
         <v>5</v>
       </c>
       <c r="U9" t="s">
-        <v>219</v>
+        <v>389</v>
       </c>
       <c r="V9">
         <v>0</v>
       </c>
       <c r="W9" t="s">
-        <v>219</v>
+        <v>389</v>
       </c>
       <c r="X9" t="s">
-        <v>219</v>
+        <v>389</v>
       </c>
       <c r="Y9" t="s">
-        <v>251</v>
+        <v>421</v>
       </c>
       <c r="AC9">
         <v>100000</v>
@@ -4876,13 +7680,13 @@
         <v>6800</v>
       </c>
       <c r="AN9" t="s">
-        <v>257</v>
+        <v>427</v>
       </c>
       <c r="AO9" t="s">
-        <v>222</v>
+        <v>392</v>
       </c>
       <c r="AQ9" t="s">
-        <v>223</v>
+        <v>393</v>
       </c>
     </row>
     <row r="10" spans="5:25" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Add discontinued 2015–2023 models (16 brands, 125 models)
Gemini research from archived brand pages, reviewed by Core. Adds
Chevrolet, Subaru, Kia and older models people still insure (Jazz,
C-HR, Sienta, March, Note, Sylphy, Colorado, Ciaz, ...). H-1 and Grand
Starex merged; Levorg dropped (no price). Prices remain unverified: a
spot check found 3 of 5 not on the cited archive page; they only feed
hidden estimates and must be verified before prices are switched on.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/examples/product-import-example.xlsx
+++ b/docs/examples/product-import-example.xlsx
@@ -568,7 +568,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1154" uniqueCount="428">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1406" uniqueCount="509">
   <si>
     <t>Unlimit Insure — แม่แบบนำเข้าข้อมูลแพ็กเกจ</t>
   </si>
@@ -1711,6 +1711,249 @@
   </si>
   <si>
     <t>Model Y</t>
+  </si>
+  <si>
+    <t>toyota-c-hr-hev</t>
+  </si>
+  <si>
+    <t>C-HR Hybrid</t>
+  </si>
+  <si>
+    <t>toyota-c-hr-ice</t>
+  </si>
+  <si>
+    <t>C-HR</t>
+  </si>
+  <si>
+    <t>toyota-sienta</t>
+  </si>
+  <si>
+    <t>Sienta</t>
+  </si>
+  <si>
+    <t>toyota-avanza</t>
+  </si>
+  <si>
+    <t>Avanza</t>
+  </si>
+  <si>
+    <t>honda-jazz</t>
+  </si>
+  <si>
+    <t>Jazz</t>
+  </si>
+  <si>
+    <t>honda-civic-hatchback</t>
+  </si>
+  <si>
+    <t>Civic Hatchback</t>
+  </si>
+  <si>
+    <t>honda-mobilio</t>
+  </si>
+  <si>
+    <t>Mobilio</t>
+  </si>
+  <si>
+    <t>honda-brio</t>
+  </si>
+  <si>
+    <t>Brio</t>
+  </si>
+  <si>
+    <t>honda-brio-amaze</t>
+  </si>
+  <si>
+    <t>Brio Amaze</t>
+  </si>
+  <si>
+    <t>mitsubishi-lancer-ex</t>
+  </si>
+  <si>
+    <t>Lancer EX</t>
+  </si>
+  <si>
+    <t>nissan-sylphy</t>
+  </si>
+  <si>
+    <t>Sylphy</t>
+  </si>
+  <si>
+    <t>nissan-march</t>
+  </si>
+  <si>
+    <t>March</t>
+  </si>
+  <si>
+    <t>nissan-note</t>
+  </si>
+  <si>
+    <t>Note</t>
+  </si>
+  <si>
+    <t>nissan-teana</t>
+  </si>
+  <si>
+    <t>Teana</t>
+  </si>
+  <si>
+    <t>nissan-x-trail-ice</t>
+  </si>
+  <si>
+    <t>X-Trail</t>
+  </si>
+  <si>
+    <t>nissan-x-trail-hev</t>
+  </si>
+  <si>
+    <t>X-Trail Hybrid</t>
+  </si>
+  <si>
+    <t>ford-fiesta</t>
+  </si>
+  <si>
+    <t>Fiesta</t>
+  </si>
+  <si>
+    <t>ford-ecosport</t>
+  </si>
+  <si>
+    <t>EcoSport</t>
+  </si>
+  <si>
+    <t>ford-focus</t>
+  </si>
+  <si>
+    <t>Focus</t>
+  </si>
+  <si>
+    <t>mg-gs</t>
+  </si>
+  <si>
+    <t>GS</t>
+  </si>
+  <si>
+    <t>mg-3-ice</t>
+  </si>
+  <si>
+    <t>MG3</t>
+  </si>
+  <si>
+    <t>mg-6</t>
+  </si>
+  <si>
+    <t>MG6</t>
+  </si>
+  <si>
+    <t>mg-v80</t>
+  </si>
+  <si>
+    <t>V80</t>
+  </si>
+  <si>
+    <t>byd-e6-ev</t>
+  </si>
+  <si>
+    <t>e6</t>
+  </si>
+  <si>
+    <t>suzuki-ciaz</t>
+  </si>
+  <si>
+    <t>Ciaz</t>
+  </si>
+  <si>
+    <t>suzuki-ertiga-ice</t>
+  </si>
+  <si>
+    <t>Ertiga</t>
+  </si>
+  <si>
+    <t>hyundai-h-1</t>
+  </si>
+  <si>
+    <t>H-1 / Grand Starex</t>
+  </si>
+  <si>
+    <t>hyundai-ioniq-ev</t>
+  </si>
+  <si>
+    <t>IONIQ Electric</t>
+  </si>
+  <si>
+    <t>hyundai-kona-ev</t>
+  </si>
+  <si>
+    <t>Kona Electric</t>
+  </si>
+  <si>
+    <t>chevrolet</t>
+  </si>
+  <si>
+    <t>Chevrolet</t>
+  </si>
+  <si>
+    <t>เชฟโรเลต</t>
+  </si>
+  <si>
+    <t>chevrolet-colorado</t>
+  </si>
+  <si>
+    <t>Colorado</t>
+  </si>
+  <si>
+    <t>chevrolet-trailblazer</t>
+  </si>
+  <si>
+    <t>Trailblazer</t>
+  </si>
+  <si>
+    <t>chevrolet-captiva</t>
+  </si>
+  <si>
+    <t>Captiva</t>
+  </si>
+  <si>
+    <t>chevrolet-cruze</t>
+  </si>
+  <si>
+    <t>Cruze</t>
+  </si>
+  <si>
+    <t>subaru</t>
+  </si>
+  <si>
+    <t>Subaru</t>
+  </si>
+  <si>
+    <t>ซูบารุ</t>
+  </si>
+  <si>
+    <t>subaru-xv</t>
+  </si>
+  <si>
+    <t>XV</t>
+  </si>
+  <si>
+    <t>kia</t>
+  </si>
+  <si>
+    <t>Kia</t>
+  </si>
+  <si>
+    <t>เกีย</t>
+  </si>
+  <si>
+    <t>kia-grand-carnival</t>
+  </si>
+  <si>
+    <t>Grand Carnival</t>
+  </si>
+  <si>
+    <t>kia-soul-ev</t>
+  </si>
+  <si>
+    <t>Soul EV</t>
   </si>
   <si>
     <t>a-type1-dealer</t>
@@ -6267,42 +6510,1158 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="91" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="92" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="93" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="94" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="95" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="96" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="97" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="98" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="99" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="100" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="101" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="102" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="103" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="104" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="105" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="106" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="107" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="108" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="109" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="110" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="111" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="112" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="113" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="114" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="115" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="116" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="117" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="118" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="119" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="120" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="121" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="122" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="123" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="124" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="125" spans="6:7" x14ac:dyDescent="0.25"/>
-    <row r="126" spans="6:7" x14ac:dyDescent="0.25"/>
+    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>155</v>
+      </c>
+      <c r="B91" t="s">
+        <v>156</v>
+      </c>
+      <c r="C91" t="s">
+        <v>157</v>
+      </c>
+      <c r="D91" t="s">
+        <v>381</v>
+      </c>
+      <c r="E91" t="s">
+        <v>382</v>
+      </c>
+      <c r="F91" t="s">
+        <v>167</v>
+      </c>
+      <c r="G91" t="s">
+        <v>168</v>
+      </c>
+      <c r="H91">
+        <v>1069000</v>
+      </c>
+      <c r="I91">
+        <v>2018</v>
+      </c>
+      <c r="J91">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>155</v>
+      </c>
+      <c r="B92" t="s">
+        <v>156</v>
+      </c>
+      <c r="C92" t="s">
+        <v>157</v>
+      </c>
+      <c r="D92" t="s">
+        <v>383</v>
+      </c>
+      <c r="E92" t="s">
+        <v>384</v>
+      </c>
+      <c r="F92" t="s">
+        <v>167</v>
+      </c>
+      <c r="G92" t="s">
+        <v>161</v>
+      </c>
+      <c r="H92">
+        <v>979000</v>
+      </c>
+      <c r="I92">
+        <v>2018</v>
+      </c>
+      <c r="J92">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>155</v>
+      </c>
+      <c r="B93" t="s">
+        <v>156</v>
+      </c>
+      <c r="C93" t="s">
+        <v>157</v>
+      </c>
+      <c r="D93" t="s">
+        <v>385</v>
+      </c>
+      <c r="E93" t="s">
+        <v>386</v>
+      </c>
+      <c r="F93" t="s">
+        <v>186</v>
+      </c>
+      <c r="G93" t="s">
+        <v>161</v>
+      </c>
+      <c r="H93">
+        <v>765000</v>
+      </c>
+      <c r="I93">
+        <v>2016</v>
+      </c>
+      <c r="J93">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>155</v>
+      </c>
+      <c r="B94" t="s">
+        <v>156</v>
+      </c>
+      <c r="C94" t="s">
+        <v>157</v>
+      </c>
+      <c r="D94" t="s">
+        <v>387</v>
+      </c>
+      <c r="E94" t="s">
+        <v>388</v>
+      </c>
+      <c r="F94" t="s">
+        <v>186</v>
+      </c>
+      <c r="G94" t="s">
+        <v>161</v>
+      </c>
+      <c r="H94">
+        <v>649000</v>
+      </c>
+      <c r="I94">
+        <v>2015</v>
+      </c>
+      <c r="J94">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>192</v>
+      </c>
+      <c r="B95" t="s">
+        <v>193</v>
+      </c>
+      <c r="C95" t="s">
+        <v>194</v>
+      </c>
+      <c r="D95" t="s">
+        <v>389</v>
+      </c>
+      <c r="E95" t="s">
+        <v>390</v>
+      </c>
+      <c r="F95" t="s">
+        <v>164</v>
+      </c>
+      <c r="G95" t="s">
+        <v>161</v>
+      </c>
+      <c r="H95">
+        <v>555000</v>
+      </c>
+      <c r="I95">
+        <v>2015</v>
+      </c>
+      <c r="J95">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>192</v>
+      </c>
+      <c r="B96" t="s">
+        <v>193</v>
+      </c>
+      <c r="C96" t="s">
+        <v>194</v>
+      </c>
+      <c r="D96" t="s">
+        <v>391</v>
+      </c>
+      <c r="E96" t="s">
+        <v>392</v>
+      </c>
+      <c r="F96" t="s">
+        <v>164</v>
+      </c>
+      <c r="G96" t="s">
+        <v>161</v>
+      </c>
+      <c r="H96">
+        <v>1169000</v>
+      </c>
+      <c r="I96">
+        <v>2017</v>
+      </c>
+      <c r="J96">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="97" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>192</v>
+      </c>
+      <c r="B97" t="s">
+        <v>193</v>
+      </c>
+      <c r="C97" t="s">
+        <v>194</v>
+      </c>
+      <c r="D97" t="s">
+        <v>393</v>
+      </c>
+      <c r="E97" t="s">
+        <v>394</v>
+      </c>
+      <c r="F97" t="s">
+        <v>186</v>
+      </c>
+      <c r="G97" t="s">
+        <v>161</v>
+      </c>
+      <c r="H97">
+        <v>659000</v>
+      </c>
+      <c r="I97">
+        <v>2015</v>
+      </c>
+      <c r="J97">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="98" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>192</v>
+      </c>
+      <c r="B98" t="s">
+        <v>193</v>
+      </c>
+      <c r="C98" t="s">
+        <v>194</v>
+      </c>
+      <c r="D98" t="s">
+        <v>395</v>
+      </c>
+      <c r="E98" t="s">
+        <v>396</v>
+      </c>
+      <c r="F98" t="s">
+        <v>164</v>
+      </c>
+      <c r="G98" t="s">
+        <v>161</v>
+      </c>
+      <c r="H98">
+        <v>495000</v>
+      </c>
+      <c r="I98">
+        <v>2015</v>
+      </c>
+      <c r="J98">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>192</v>
+      </c>
+      <c r="B99" t="s">
+        <v>193</v>
+      </c>
+      <c r="C99" t="s">
+        <v>194</v>
+      </c>
+      <c r="D99" t="s">
+        <v>397</v>
+      </c>
+      <c r="E99" t="s">
+        <v>398</v>
+      </c>
+      <c r="F99" t="s">
+        <v>160</v>
+      </c>
+      <c r="G99" t="s">
+        <v>161</v>
+      </c>
+      <c r="H99">
+        <v>517000</v>
+      </c>
+      <c r="I99">
+        <v>2015</v>
+      </c>
+      <c r="J99">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>224</v>
+      </c>
+      <c r="B100" t="s">
+        <v>225</v>
+      </c>
+      <c r="C100" t="s">
+        <v>226</v>
+      </c>
+      <c r="D100" t="s">
+        <v>399</v>
+      </c>
+      <c r="E100" t="s">
+        <v>400</v>
+      </c>
+      <c r="F100" t="s">
+        <v>160</v>
+      </c>
+      <c r="G100" t="s">
+        <v>161</v>
+      </c>
+      <c r="H100">
+        <v>879000</v>
+      </c>
+      <c r="I100">
+        <v>2015</v>
+      </c>
+      <c r="J100">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>239</v>
+      </c>
+      <c r="B101" t="s">
+        <v>240</v>
+      </c>
+      <c r="C101" t="s">
+        <v>241</v>
+      </c>
+      <c r="D101" t="s">
+        <v>401</v>
+      </c>
+      <c r="E101" t="s">
+        <v>402</v>
+      </c>
+      <c r="F101" t="s">
+        <v>160</v>
+      </c>
+      <c r="G101" t="s">
+        <v>161</v>
+      </c>
+      <c r="H101">
+        <v>833000</v>
+      </c>
+      <c r="I101">
+        <v>2015</v>
+      </c>
+      <c r="J101">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>239</v>
+      </c>
+      <c r="B102" t="s">
+        <v>240</v>
+      </c>
+      <c r="C102" t="s">
+        <v>241</v>
+      </c>
+      <c r="D102" t="s">
+        <v>403</v>
+      </c>
+      <c r="E102" t="s">
+        <v>404</v>
+      </c>
+      <c r="F102" t="s">
+        <v>164</v>
+      </c>
+      <c r="G102" t="s">
+        <v>161</v>
+      </c>
+      <c r="H102">
+        <v>420000</v>
+      </c>
+      <c r="I102">
+        <v>2015</v>
+      </c>
+      <c r="J102">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="103" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>239</v>
+      </c>
+      <c r="B103" t="s">
+        <v>240</v>
+      </c>
+      <c r="C103" t="s">
+        <v>241</v>
+      </c>
+      <c r="D103" t="s">
+        <v>405</v>
+      </c>
+      <c r="E103" t="s">
+        <v>406</v>
+      </c>
+      <c r="F103" t="s">
+        <v>164</v>
+      </c>
+      <c r="G103" t="s">
+        <v>161</v>
+      </c>
+      <c r="H103">
+        <v>530000</v>
+      </c>
+      <c r="I103">
+        <v>2017</v>
+      </c>
+      <c r="J103">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="104" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>239</v>
+      </c>
+      <c r="B104" t="s">
+        <v>240</v>
+      </c>
+      <c r="C104" t="s">
+        <v>241</v>
+      </c>
+      <c r="D104" t="s">
+        <v>407</v>
+      </c>
+      <c r="E104" t="s">
+        <v>408</v>
+      </c>
+      <c r="F104" t="s">
+        <v>160</v>
+      </c>
+      <c r="G104" t="s">
+        <v>161</v>
+      </c>
+      <c r="H104">
+        <v>1339000</v>
+      </c>
+      <c r="I104">
+        <v>2015</v>
+      </c>
+      <c r="J104">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="105" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>239</v>
+      </c>
+      <c r="B105" t="s">
+        <v>240</v>
+      </c>
+      <c r="C105" t="s">
+        <v>241</v>
+      </c>
+      <c r="D105" t="s">
+        <v>409</v>
+      </c>
+      <c r="E105" t="s">
+        <v>410</v>
+      </c>
+      <c r="F105" t="s">
+        <v>167</v>
+      </c>
+      <c r="G105" t="s">
+        <v>161</v>
+      </c>
+      <c r="H105">
+        <v>1350000</v>
+      </c>
+      <c r="I105">
+        <v>2015</v>
+      </c>
+      <c r="J105">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>239</v>
+      </c>
+      <c r="B106" t="s">
+        <v>240</v>
+      </c>
+      <c r="C106" t="s">
+        <v>241</v>
+      </c>
+      <c r="D106" t="s">
+        <v>411</v>
+      </c>
+      <c r="E106" t="s">
+        <v>412</v>
+      </c>
+      <c r="F106" t="s">
+        <v>167</v>
+      </c>
+      <c r="G106" t="s">
+        <v>168</v>
+      </c>
+      <c r="H106">
+        <v>1537000</v>
+      </c>
+      <c r="I106">
+        <v>2015</v>
+      </c>
+      <c r="J106">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>271</v>
+      </c>
+      <c r="B107" t="s">
+        <v>272</v>
+      </c>
+      <c r="C107" t="s">
+        <v>273</v>
+      </c>
+      <c r="D107" t="s">
+        <v>413</v>
+      </c>
+      <c r="E107" t="s">
+        <v>414</v>
+      </c>
+      <c r="F107" t="s">
+        <v>164</v>
+      </c>
+      <c r="G107" t="s">
+        <v>161</v>
+      </c>
+      <c r="H107">
+        <v>644000</v>
+      </c>
+      <c r="I107">
+        <v>2015</v>
+      </c>
+      <c r="J107">
+        <v>2019</v>
+      </c>
+    </row>
+    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>271</v>
+      </c>
+      <c r="B108" t="s">
+        <v>272</v>
+      </c>
+      <c r="C108" t="s">
+        <v>273</v>
+      </c>
+      <c r="D108" t="s">
+        <v>415</v>
+      </c>
+      <c r="E108" t="s">
+        <v>416</v>
+      </c>
+      <c r="F108" t="s">
+        <v>167</v>
+      </c>
+      <c r="G108" t="s">
+        <v>161</v>
+      </c>
+      <c r="H108">
+        <v>739000</v>
+      </c>
+      <c r="I108">
+        <v>2015</v>
+      </c>
+      <c r="J108">
+        <v>2019</v>
+      </c>
+    </row>
+    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>271</v>
+      </c>
+      <c r="B109" t="s">
+        <v>272</v>
+      </c>
+      <c r="C109" t="s">
+        <v>273</v>
+      </c>
+      <c r="D109" t="s">
+        <v>417</v>
+      </c>
+      <c r="E109" t="s">
+        <v>418</v>
+      </c>
+      <c r="F109" t="s">
+        <v>160</v>
+      </c>
+      <c r="G109" t="s">
+        <v>161</v>
+      </c>
+      <c r="H109">
+        <v>1099000</v>
+      </c>
+      <c r="I109">
+        <v>2015</v>
+      </c>
+      <c r="J109">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>280</v>
+      </c>
+      <c r="B110" t="s">
+        <v>281</v>
+      </c>
+      <c r="C110" t="s">
+        <v>282</v>
+      </c>
+      <c r="D110" t="s">
+        <v>419</v>
+      </c>
+      <c r="E110" t="s">
+        <v>420</v>
+      </c>
+      <c r="F110" t="s">
+        <v>167</v>
+      </c>
+      <c r="G110" t="s">
+        <v>161</v>
+      </c>
+      <c r="H110">
+        <v>890000</v>
+      </c>
+      <c r="I110">
+        <v>2016</v>
+      </c>
+      <c r="J110">
+        <v>2019</v>
+      </c>
+    </row>
+    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>280</v>
+      </c>
+      <c r="B111" t="s">
+        <v>281</v>
+      </c>
+      <c r="C111" t="s">
+        <v>282</v>
+      </c>
+      <c r="D111" t="s">
+        <v>421</v>
+      </c>
+      <c r="E111" t="s">
+        <v>422</v>
+      </c>
+      <c r="F111" t="s">
+        <v>164</v>
+      </c>
+      <c r="G111" t="s">
+        <v>161</v>
+      </c>
+      <c r="H111">
+        <v>519000</v>
+      </c>
+      <c r="I111">
+        <v>2015</v>
+      </c>
+      <c r="J111">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>280</v>
+      </c>
+      <c r="B112" t="s">
+        <v>281</v>
+      </c>
+      <c r="C112" t="s">
+        <v>282</v>
+      </c>
+      <c r="D112" t="s">
+        <v>423</v>
+      </c>
+      <c r="E112" t="s">
+        <v>424</v>
+      </c>
+      <c r="F112" t="s">
+        <v>160</v>
+      </c>
+      <c r="G112" t="s">
+        <v>161</v>
+      </c>
+      <c r="H112">
+        <v>898000</v>
+      </c>
+      <c r="I112">
+        <v>2015</v>
+      </c>
+      <c r="J112">
+        <v>2019</v>
+      </c>
+    </row>
+    <row r="113" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>280</v>
+      </c>
+      <c r="B113" t="s">
+        <v>281</v>
+      </c>
+      <c r="C113" t="s">
+        <v>282</v>
+      </c>
+      <c r="D113" t="s">
+        <v>425</v>
+      </c>
+      <c r="E113" t="s">
+        <v>426</v>
+      </c>
+      <c r="F113" t="s">
+        <v>186</v>
+      </c>
+      <c r="G113" t="s">
+        <v>161</v>
+      </c>
+      <c r="H113">
+        <v>988000</v>
+      </c>
+      <c r="I113">
+        <v>2019</v>
+      </c>
+      <c r="J113">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="114" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>308</v>
+      </c>
+      <c r="B114" t="s">
+        <v>309</v>
+      </c>
+      <c r="C114" t="s">
+        <v>310</v>
+      </c>
+      <c r="D114" t="s">
+        <v>427</v>
+      </c>
+      <c r="E114" t="s">
+        <v>428</v>
+      </c>
+      <c r="F114" t="s">
+        <v>186</v>
+      </c>
+      <c r="G114" t="s">
+        <v>191</v>
+      </c>
+      <c r="H114">
+        <v>1890000</v>
+      </c>
+      <c r="I114">
+        <v>2018</v>
+      </c>
+      <c r="J114">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="115" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>323</v>
+      </c>
+      <c r="B115" t="s">
+        <v>324</v>
+      </c>
+      <c r="C115" t="s">
+        <v>325</v>
+      </c>
+      <c r="D115" t="s">
+        <v>429</v>
+      </c>
+      <c r="E115" t="s">
+        <v>430</v>
+      </c>
+      <c r="F115" t="s">
+        <v>160</v>
+      </c>
+      <c r="G115" t="s">
+        <v>161</v>
+      </c>
+      <c r="H115">
+        <v>528000</v>
+      </c>
+      <c r="I115">
+        <v>2015</v>
+      </c>
+      <c r="J115">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="116" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>323</v>
+      </c>
+      <c r="B116" t="s">
+        <v>324</v>
+      </c>
+      <c r="C116" t="s">
+        <v>325</v>
+      </c>
+      <c r="D116" t="s">
+        <v>431</v>
+      </c>
+      <c r="E116" t="s">
+        <v>432</v>
+      </c>
+      <c r="F116" t="s">
+        <v>186</v>
+      </c>
+      <c r="G116" t="s">
+        <v>161</v>
+      </c>
+      <c r="H116">
+        <v>658000</v>
+      </c>
+      <c r="I116">
+        <v>2015</v>
+      </c>
+      <c r="J116">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="117" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>357</v>
+      </c>
+      <c r="B117" t="s">
+        <v>358</v>
+      </c>
+      <c r="C117" t="s">
+        <v>359</v>
+      </c>
+      <c r="D117" t="s">
+        <v>433</v>
+      </c>
+      <c r="E117" t="s">
+        <v>434</v>
+      </c>
+      <c r="F117" t="s">
+        <v>186</v>
+      </c>
+      <c r="G117" t="s">
+        <v>161</v>
+      </c>
+      <c r="H117">
+        <v>1329000</v>
+      </c>
+      <c r="I117">
+        <v>2015</v>
+      </c>
+      <c r="J117">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="118" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>357</v>
+      </c>
+      <c r="B118" t="s">
+        <v>358</v>
+      </c>
+      <c r="C118" t="s">
+        <v>359</v>
+      </c>
+      <c r="D118" t="s">
+        <v>435</v>
+      </c>
+      <c r="E118" t="s">
+        <v>436</v>
+      </c>
+      <c r="F118" t="s">
+        <v>164</v>
+      </c>
+      <c r="G118" t="s">
+        <v>191</v>
+      </c>
+      <c r="H118">
+        <v>1749000</v>
+      </c>
+      <c r="I118">
+        <v>2019</v>
+      </c>
+      <c r="J118">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="119" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>357</v>
+      </c>
+      <c r="B119" t="s">
+        <v>358</v>
+      </c>
+      <c r="C119" t="s">
+        <v>359</v>
+      </c>
+      <c r="D119" t="s">
+        <v>437</v>
+      </c>
+      <c r="E119" t="s">
+        <v>438</v>
+      </c>
+      <c r="F119" t="s">
+        <v>167</v>
+      </c>
+      <c r="G119" t="s">
+        <v>191</v>
+      </c>
+      <c r="H119">
+        <v>1849000</v>
+      </c>
+      <c r="I119">
+        <v>2019</v>
+      </c>
+      <c r="J119">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="120" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>439</v>
+      </c>
+      <c r="B120" t="s">
+        <v>440</v>
+      </c>
+      <c r="C120" t="s">
+        <v>441</v>
+      </c>
+      <c r="D120" t="s">
+        <v>442</v>
+      </c>
+      <c r="E120" t="s">
+        <v>443</v>
+      </c>
+      <c r="F120" t="s">
+        <v>181</v>
+      </c>
+      <c r="G120" t="s">
+        <v>161</v>
+      </c>
+      <c r="H120">
+        <v>538000</v>
+      </c>
+      <c r="I120">
+        <v>2015</v>
+      </c>
+      <c r="J120">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="121" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>439</v>
+      </c>
+      <c r="B121" t="s">
+        <v>440</v>
+      </c>
+      <c r="C121" t="s">
+        <v>441</v>
+      </c>
+      <c r="D121" t="s">
+        <v>444</v>
+      </c>
+      <c r="E121" t="s">
+        <v>445</v>
+      </c>
+      <c r="F121" t="s">
+        <v>167</v>
+      </c>
+      <c r="G121" t="s">
+        <v>161</v>
+      </c>
+      <c r="H121">
+        <v>1144000</v>
+      </c>
+      <c r="I121">
+        <v>2015</v>
+      </c>
+      <c r="J121">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="122" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>439</v>
+      </c>
+      <c r="B122" t="s">
+        <v>440</v>
+      </c>
+      <c r="C122" t="s">
+        <v>441</v>
+      </c>
+      <c r="D122" t="s">
+        <v>446</v>
+      </c>
+      <c r="E122" t="s">
+        <v>447</v>
+      </c>
+      <c r="F122" t="s">
+        <v>167</v>
+      </c>
+      <c r="G122" t="s">
+        <v>161</v>
+      </c>
+      <c r="H122">
+        <v>999000</v>
+      </c>
+      <c r="I122">
+        <v>2015</v>
+      </c>
+      <c r="J122">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="123" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>439</v>
+      </c>
+      <c r="B123" t="s">
+        <v>440</v>
+      </c>
+      <c r="C123" t="s">
+        <v>441</v>
+      </c>
+      <c r="D123" t="s">
+        <v>448</v>
+      </c>
+      <c r="E123" t="s">
+        <v>449</v>
+      </c>
+      <c r="F123" t="s">
+        <v>160</v>
+      </c>
+      <c r="G123" t="s">
+        <v>161</v>
+      </c>
+      <c r="H123">
+        <v>946000</v>
+      </c>
+      <c r="I123">
+        <v>2015</v>
+      </c>
+      <c r="J123">
+        <v>2017</v>
+      </c>
+    </row>
+    <row r="124" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>450</v>
+      </c>
+      <c r="B124" t="s">
+        <v>451</v>
+      </c>
+      <c r="C124" t="s">
+        <v>452</v>
+      </c>
+      <c r="D124" t="s">
+        <v>453</v>
+      </c>
+      <c r="E124" t="s">
+        <v>454</v>
+      </c>
+      <c r="F124" t="s">
+        <v>167</v>
+      </c>
+      <c r="G124" t="s">
+        <v>161</v>
+      </c>
+      <c r="H124">
+        <v>1159000</v>
+      </c>
+      <c r="I124">
+        <v>2015</v>
+      </c>
+      <c r="J124">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="125" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>455</v>
+      </c>
+      <c r="B125" t="s">
+        <v>456</v>
+      </c>
+      <c r="C125" t="s">
+        <v>457</v>
+      </c>
+      <c r="D125" t="s">
+        <v>458</v>
+      </c>
+      <c r="E125" t="s">
+        <v>459</v>
+      </c>
+      <c r="F125" t="s">
+        <v>186</v>
+      </c>
+      <c r="G125" t="s">
+        <v>161</v>
+      </c>
+      <c r="H125">
+        <v>1397000</v>
+      </c>
+      <c r="I125">
+        <v>2015</v>
+      </c>
+      <c r="J125">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="126" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
+        <v>455</v>
+      </c>
+      <c r="B126" t="s">
+        <v>456</v>
+      </c>
+      <c r="C126" t="s">
+        <v>457</v>
+      </c>
+      <c r="D126" t="s">
+        <v>460</v>
+      </c>
+      <c r="E126" t="s">
+        <v>461</v>
+      </c>
+      <c r="F126" t="s">
+        <v>164</v>
+      </c>
+      <c r="G126" t="s">
+        <v>191</v>
+      </c>
+      <c r="H126">
+        <v>2387000</v>
+      </c>
+      <c r="I126">
+        <v>2018</v>
+      </c>
+      <c r="J126">
+        <v>2021</v>
+      </c>
+    </row>
     <row r="127" spans="6:7" x14ac:dyDescent="0.25"/>
     <row r="128" spans="6:7" x14ac:dyDescent="0.25"/>
     <row r="129" spans="6:7" x14ac:dyDescent="0.25"/>
@@ -6877,40 +8236,40 @@
         <v>143</v>
       </c>
       <c r="B2" t="s">
-        <v>381</v>
+        <v>462</v>
       </c>
       <c r="C2" t="s">
-        <v>382</v>
+        <v>463</v>
       </c>
       <c r="D2" t="s">
-        <v>383</v>
+        <v>464</v>
       </c>
       <c r="E2" t="s">
-        <v>384</v>
+        <v>465</v>
       </c>
       <c r="F2" t="s">
-        <v>385</v>
+        <v>466</v>
       </c>
       <c r="G2" t="s">
-        <v>386</v>
+        <v>467</v>
       </c>
       <c r="H2" t="s">
-        <v>387</v>
+        <v>468</v>
       </c>
       <c r="I2">
         <v>0</v>
       </c>
       <c r="J2" t="s">
-        <v>388</v>
+        <v>469</v>
       </c>
       <c r="K2" t="s">
-        <v>388</v>
+        <v>469</v>
       </c>
       <c r="L2" t="s">
-        <v>388</v>
+        <v>469</v>
       </c>
       <c r="M2" t="s">
-        <v>388</v>
+        <v>469</v>
       </c>
       <c r="N2">
         <v>1000000</v>
@@ -6934,16 +8293,16 @@
         <v>5</v>
       </c>
       <c r="U2" t="s">
-        <v>388</v>
+        <v>469</v>
       </c>
       <c r="V2">
         <v>0</v>
       </c>
       <c r="W2" t="s">
-        <v>389</v>
+        <v>470</v>
       </c>
       <c r="X2" t="s">
-        <v>389</v>
+        <v>470</v>
       </c>
       <c r="Y2" t="s">
         <v>105</v>
@@ -6961,16 +8320,16 @@
         <v>5</v>
       </c>
       <c r="AM2" t="s">
-        <v>390</v>
+        <v>471</v>
       </c>
       <c r="AN2" t="s">
-        <v>391</v>
+        <v>472</v>
       </c>
       <c r="AO2" t="s">
-        <v>392</v>
+        <v>473</v>
       </c>
       <c r="AQ2" t="s">
-        <v>393</v>
+        <v>474</v>
       </c>
     </row>
     <row r="3" spans="1:43" x14ac:dyDescent="0.25">
@@ -6978,40 +8337,40 @@
         <v>143</v>
       </c>
       <c r="B3" t="s">
-        <v>381</v>
+        <v>462</v>
       </c>
       <c r="C3" t="s">
-        <v>382</v>
+        <v>463</v>
       </c>
       <c r="D3" t="s">
-        <v>383</v>
+        <v>464</v>
       </c>
       <c r="E3" t="s">
-        <v>384</v>
+        <v>465</v>
       </c>
       <c r="F3" t="s">
-        <v>394</v>
+        <v>475</v>
       </c>
       <c r="G3" t="s">
-        <v>395</v>
+        <v>476</v>
       </c>
       <c r="H3" t="s">
-        <v>387</v>
+        <v>468</v>
       </c>
       <c r="I3">
         <v>0</v>
       </c>
       <c r="J3" t="s">
-        <v>388</v>
+        <v>469</v>
       </c>
       <c r="K3" t="s">
-        <v>388</v>
+        <v>469</v>
       </c>
       <c r="L3" t="s">
-        <v>388</v>
+        <v>469</v>
       </c>
       <c r="M3" t="s">
-        <v>388</v>
+        <v>469</v>
       </c>
       <c r="N3">
         <v>1000000</v>
@@ -7035,16 +8394,16 @@
         <v>5</v>
       </c>
       <c r="U3" t="s">
-        <v>388</v>
+        <v>469</v>
       </c>
       <c r="V3">
         <v>0</v>
       </c>
       <c r="W3" t="s">
-        <v>389</v>
+        <v>470</v>
       </c>
       <c r="X3" t="s">
-        <v>389</v>
+        <v>470</v>
       </c>
       <c r="Y3" t="s">
         <v>105</v>
@@ -7062,16 +8421,16 @@
         <v>5</v>
       </c>
       <c r="AM3" t="s">
-        <v>396</v>
+        <v>477</v>
       </c>
       <c r="AN3" t="s">
-        <v>397</v>
+        <v>478</v>
       </c>
       <c r="AO3" t="s">
-        <v>392</v>
+        <v>473</v>
       </c>
       <c r="AQ3" t="s">
-        <v>393</v>
+        <v>474</v>
       </c>
     </row>
     <row r="4" spans="1:43" x14ac:dyDescent="0.25">
@@ -7079,40 +8438,40 @@
         <v>147</v>
       </c>
       <c r="B4" t="s">
-        <v>398</v>
+        <v>479</v>
       </c>
       <c r="C4" t="s">
-        <v>399</v>
+        <v>480</v>
       </c>
       <c r="D4" t="s">
-        <v>400</v>
+        <v>481</v>
       </c>
       <c r="E4" t="s">
-        <v>384</v>
+        <v>465</v>
       </c>
       <c r="F4" t="s">
-        <v>385</v>
+        <v>466</v>
       </c>
       <c r="G4" t="s">
-        <v>395</v>
+        <v>476</v>
       </c>
       <c r="H4" t="s">
-        <v>401</v>
+        <v>482</v>
       </c>
       <c r="I4">
         <v>2000</v>
       </c>
       <c r="J4" t="s">
-        <v>388</v>
+        <v>469</v>
       </c>
       <c r="K4" t="s">
-        <v>388</v>
+        <v>469</v>
       </c>
       <c r="L4" t="s">
-        <v>388</v>
+        <v>469</v>
       </c>
       <c r="M4" t="s">
-        <v>388</v>
+        <v>469</v>
       </c>
       <c r="N4">
         <v>1000000</v>
@@ -7136,16 +8495,16 @@
         <v>5</v>
       </c>
       <c r="U4" t="s">
-        <v>388</v>
+        <v>469</v>
       </c>
       <c r="V4">
         <v>0</v>
       </c>
       <c r="W4" t="s">
-        <v>389</v>
+        <v>470</v>
       </c>
       <c r="X4" t="s">
-        <v>389</v>
+        <v>470</v>
       </c>
       <c r="Y4" t="s">
         <v>105</v>
@@ -7163,16 +8522,16 @@
         <v>12</v>
       </c>
       <c r="AM4" t="s">
-        <v>390</v>
+        <v>471</v>
       </c>
       <c r="AN4" t="s">
-        <v>402</v>
+        <v>483</v>
       </c>
       <c r="AO4" t="s">
-        <v>392</v>
+        <v>473</v>
       </c>
       <c r="AQ4" t="s">
-        <v>393</v>
+        <v>474</v>
       </c>
     </row>
     <row r="5" spans="1:43" x14ac:dyDescent="0.25">
@@ -7180,40 +8539,40 @@
         <v>151</v>
       </c>
       <c r="B5" t="s">
-        <v>403</v>
+        <v>484</v>
       </c>
       <c r="C5" t="s">
-        <v>404</v>
+        <v>485</v>
       </c>
       <c r="D5" t="s">
-        <v>405</v>
+        <v>486</v>
       </c>
       <c r="E5" t="s">
-        <v>384</v>
+        <v>465</v>
       </c>
       <c r="F5" t="s">
-        <v>385</v>
+        <v>466</v>
       </c>
       <c r="G5" t="s">
-        <v>395</v>
+        <v>476</v>
       </c>
       <c r="H5" t="s">
-        <v>387</v>
+        <v>468</v>
       </c>
       <c r="I5">
         <v>0</v>
       </c>
       <c r="J5" t="s">
-        <v>388</v>
+        <v>469</v>
       </c>
       <c r="K5" t="s">
-        <v>388</v>
+        <v>469</v>
       </c>
       <c r="L5" t="s">
-        <v>388</v>
+        <v>469</v>
       </c>
       <c r="M5" t="s">
-        <v>388</v>
+        <v>469</v>
       </c>
       <c r="N5">
         <v>1000000</v>
@@ -7237,16 +8596,16 @@
         <v>5</v>
       </c>
       <c r="U5" t="s">
-        <v>388</v>
+        <v>469</v>
       </c>
       <c r="V5">
         <v>7</v>
       </c>
       <c r="W5" t="s">
-        <v>389</v>
+        <v>470</v>
       </c>
       <c r="X5" t="s">
-        <v>389</v>
+        <v>470</v>
       </c>
       <c r="Y5" t="s">
         <v>105</v>
@@ -7264,16 +8623,16 @@
         <v>7</v>
       </c>
       <c r="AM5" t="s">
-        <v>406</v>
+        <v>487</v>
       </c>
       <c r="AN5" t="s">
-        <v>407</v>
+        <v>488</v>
       </c>
       <c r="AO5" t="s">
-        <v>392</v>
+        <v>473</v>
       </c>
       <c r="AQ5" t="s">
-        <v>393</v>
+        <v>474</v>
       </c>
     </row>
     <row r="6" spans="1:43" x14ac:dyDescent="0.25">
@@ -7281,40 +8640,40 @@
         <v>151</v>
       </c>
       <c r="B6" t="s">
-        <v>408</v>
+        <v>489</v>
       </c>
       <c r="C6" t="s">
-        <v>409</v>
+        <v>490</v>
       </c>
       <c r="D6" t="s">
-        <v>410</v>
+        <v>491</v>
       </c>
       <c r="E6" t="s">
-        <v>384</v>
+        <v>465</v>
       </c>
       <c r="F6" t="s">
-        <v>385</v>
+        <v>466</v>
       </c>
       <c r="G6" t="s">
-        <v>395</v>
+        <v>476</v>
       </c>
       <c r="H6" t="s">
-        <v>401</v>
+        <v>482</v>
       </c>
       <c r="I6">
         <v>0</v>
       </c>
       <c r="J6" t="s">
-        <v>388</v>
+        <v>469</v>
       </c>
       <c r="K6" t="s">
-        <v>388</v>
+        <v>469</v>
       </c>
       <c r="L6" t="s">
-        <v>388</v>
+        <v>469</v>
       </c>
       <c r="M6" t="s">
-        <v>389</v>
+        <v>470</v>
       </c>
       <c r="N6">
         <v>1000000</v>
@@ -7338,16 +8697,16 @@
         <v>5</v>
       </c>
       <c r="U6" t="s">
-        <v>389</v>
+        <v>470</v>
       </c>
       <c r="V6">
         <v>0</v>
       </c>
       <c r="W6" t="s">
-        <v>389</v>
+        <v>470</v>
       </c>
       <c r="X6" t="s">
-        <v>389</v>
+        <v>470</v>
       </c>
       <c r="Y6" t="s">
         <v>105</v>
@@ -7365,13 +8724,13 @@
         <v>15</v>
       </c>
       <c r="AN6" t="s">
-        <v>411</v>
+        <v>492</v>
       </c>
       <c r="AO6" t="s">
-        <v>392</v>
+        <v>473</v>
       </c>
       <c r="AQ6" t="s">
-        <v>393</v>
+        <v>474</v>
       </c>
     </row>
     <row r="7" spans="1:43" x14ac:dyDescent="0.25">
@@ -7379,40 +8738,40 @@
         <v>151</v>
       </c>
       <c r="B7" t="s">
-        <v>412</v>
+        <v>493</v>
       </c>
       <c r="C7" t="s">
-        <v>413</v>
+        <v>494</v>
       </c>
       <c r="D7" t="s">
-        <v>414</v>
+        <v>495</v>
       </c>
       <c r="E7" t="s">
-        <v>384</v>
+        <v>465</v>
       </c>
       <c r="F7" t="s">
-        <v>385</v>
+        <v>466</v>
       </c>
       <c r="G7" t="s">
-        <v>395</v>
+        <v>476</v>
       </c>
       <c r="H7" t="s">
-        <v>387</v>
+        <v>468</v>
       </c>
       <c r="I7">
         <v>0</v>
       </c>
       <c r="J7" t="s">
-        <v>388</v>
+        <v>469</v>
       </c>
       <c r="K7" t="s">
-        <v>388</v>
+        <v>469</v>
       </c>
       <c r="L7" t="s">
-        <v>388</v>
+        <v>469</v>
       </c>
       <c r="M7" t="s">
-        <v>388</v>
+        <v>469</v>
       </c>
       <c r="N7">
         <v>1000000</v>
@@ -7436,16 +8795,16 @@
         <v>5</v>
       </c>
       <c r="U7" t="s">
-        <v>388</v>
+        <v>469</v>
       </c>
       <c r="V7">
         <v>5</v>
       </c>
       <c r="W7" t="s">
-        <v>388</v>
+        <v>469</v>
       </c>
       <c r="X7" t="s">
-        <v>388</v>
+        <v>469</v>
       </c>
       <c r="Y7" t="s">
         <v>105</v>
@@ -7466,16 +8825,16 @@
         <v>191</v>
       </c>
       <c r="AM7" t="s">
-        <v>415</v>
+        <v>496</v>
       </c>
       <c r="AN7" t="s">
-        <v>416</v>
+        <v>497</v>
       </c>
       <c r="AO7" t="s">
-        <v>392</v>
+        <v>473</v>
       </c>
       <c r="AQ7" t="s">
-        <v>393</v>
+        <v>474</v>
       </c>
     </row>
     <row r="8" spans="1:43" x14ac:dyDescent="0.25">
@@ -7483,40 +8842,40 @@
         <v>143</v>
       </c>
       <c r="B8" t="s">
-        <v>417</v>
+        <v>498</v>
       </c>
       <c r="C8" t="s">
-        <v>418</v>
+        <v>499</v>
       </c>
       <c r="D8" t="s">
-        <v>419</v>
+        <v>500</v>
       </c>
       <c r="E8" t="s">
-        <v>420</v>
+        <v>501</v>
       </c>
       <c r="F8" t="s">
-        <v>385</v>
+        <v>466</v>
       </c>
       <c r="G8" t="s">
-        <v>395</v>
+        <v>476</v>
       </c>
       <c r="H8" t="s">
-        <v>401</v>
+        <v>482</v>
       </c>
       <c r="I8">
         <v>0</v>
       </c>
       <c r="J8" t="s">
-        <v>388</v>
+        <v>469</v>
       </c>
       <c r="K8" t="s">
-        <v>389</v>
+        <v>470</v>
       </c>
       <c r="L8" t="s">
-        <v>388</v>
+        <v>469</v>
       </c>
       <c r="M8" t="s">
-        <v>388</v>
+        <v>469</v>
       </c>
       <c r="N8">
         <v>1000000</v>
@@ -7540,19 +8899,19 @@
         <v>5</v>
       </c>
       <c r="U8" t="s">
-        <v>388</v>
+        <v>469</v>
       </c>
       <c r="V8">
         <v>0</v>
       </c>
       <c r="W8" t="s">
-        <v>389</v>
+        <v>470</v>
       </c>
       <c r="X8" t="s">
-        <v>389</v>
+        <v>470</v>
       </c>
       <c r="Y8" t="s">
-        <v>421</v>
+        <v>502</v>
       </c>
       <c r="AC8">
         <v>200000</v>
@@ -7573,16 +8932,16 @@
         <v>9200</v>
       </c>
       <c r="AM8" t="s">
-        <v>390</v>
+        <v>471</v>
       </c>
       <c r="AN8" t="s">
-        <v>422</v>
+        <v>503</v>
       </c>
       <c r="AO8" t="s">
-        <v>392</v>
+        <v>473</v>
       </c>
       <c r="AQ8" t="s">
-        <v>393</v>
+        <v>474</v>
       </c>
     </row>
     <row r="9" spans="1:43" x14ac:dyDescent="0.25">
@@ -7590,40 +8949,40 @@
         <v>147</v>
       </c>
       <c r="B9" t="s">
-        <v>423</v>
+        <v>504</v>
       </c>
       <c r="C9" t="s">
-        <v>424</v>
+        <v>505</v>
       </c>
       <c r="D9" t="s">
-        <v>425</v>
+        <v>506</v>
       </c>
       <c r="E9" t="s">
-        <v>426</v>
+        <v>507</v>
       </c>
       <c r="F9" t="s">
-        <v>385</v>
+        <v>466</v>
       </c>
       <c r="G9" t="s">
-        <v>395</v>
+        <v>476</v>
       </c>
       <c r="H9" t="s">
-        <v>401</v>
+        <v>482</v>
       </c>
       <c r="I9">
         <v>0</v>
       </c>
       <c r="J9" t="s">
-        <v>388</v>
+        <v>469</v>
       </c>
       <c r="K9" t="s">
-        <v>389</v>
+        <v>470</v>
       </c>
       <c r="L9" t="s">
-        <v>389</v>
+        <v>470</v>
       </c>
       <c r="M9" t="s">
-        <v>389</v>
+        <v>470</v>
       </c>
       <c r="N9">
         <v>1000000</v>
@@ -7647,19 +9006,19 @@
         <v>5</v>
       </c>
       <c r="U9" t="s">
-        <v>389</v>
+        <v>470</v>
       </c>
       <c r="V9">
         <v>0</v>
       </c>
       <c r="W9" t="s">
-        <v>389</v>
+        <v>470</v>
       </c>
       <c r="X9" t="s">
-        <v>389</v>
+        <v>470</v>
       </c>
       <c r="Y9" t="s">
-        <v>421</v>
+        <v>502</v>
       </c>
       <c r="AC9">
         <v>100000</v>
@@ -7680,13 +9039,13 @@
         <v>6800</v>
       </c>
       <c r="AN9" t="s">
-        <v>427</v>
+        <v>508</v>
       </c>
       <c r="AO9" t="s">
-        <v>392</v>
+        <v>473</v>
       </c>
       <c r="AQ9" t="s">
-        <v>393</v>
+        <v>474</v>
       </c>
     </row>
     <row r="10" spans="5:25" x14ac:dyDescent="0.25"/>

</xml_diff>